<commit_message>
Rétablit la fiche de Jennifer Saul
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-autre-actif.xlsx
+++ b/data/frise-philosophes-autre-actif.xlsx
@@ -6437,7 +6437,9 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="7"/>
+      <c r="A88" s="7" t="n">
+        <v>1968</v>
+      </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7" t="s">
         <v>656</v>

</xml_diff>

<commit_message>
Met à jour la fiche de Jennifer Saul et stabilise la liste de recherche
La liste est insérée une image après le chargement des polices, pour que
leur application et l'insertion ne tombent pas dans la même image.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-autre-actif.xlsx
+++ b/data/frise-philosophes-autre-actif.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="794">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="795">
   <si>
     <t xml:space="preserve">FRISE DES PHILOSOPHES CONTEMPORAINS (AUTRES) — Données source</t>
   </si>
@@ -2276,7 +2276,34 @@
     <t xml:space="preserve">Jennifer SAUL</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Jennifer_Saul"  style="color:#6A142A"  title=" Wikipedia"&gt;Jennifer SAUL&lt;/a&gt;  est une philosophe britanique spécialisée en philosophie du langage, en philosophie féministe et en philosophie de l'esprit. Elle est connue pour ses travaux sur les &lt;a href="https://www.youtube.com/watch?v=2_FqrHs9S-s" style="color:#88A1E9" title="Jennifer Saul: 'Why Implicit Bias Matters' par The Royal Institute of Philosophy"&gt;biais implicites&lt;/a&gt; et de leur impact sur les comportements sociaux. Elle explore comment ils influencent les décisions, les interactions et les structures sociales, même en l'absence de préjugés explicites, le langage et le genre, ainsi que pour ses analyses des questions liées à la discrimination et à l'oppression. &lt;/p&gt; &lt;p&gt; Elle s'intéresse aussi à la manière dont le langage peut véhiculer des stéréotypes et renforcer des inégalités, même lorsque les locuteurs n'en ont pas conscience. Son livre "Lying, Misleading, and What Is Said" aborde notamment les questions de tromperie et de manipulation linguistique. &lt;/p&gt; &lt;p&gt; Dans son ouvrage  "Feminism: Issues &amp; Arguments", elle examine des débats clés du féminisme, comme la définition du genre, l'objectification ou les controverses autour de la pornographie et de la prostitution. Elle défend une approche analytique rigoureuse des questions féministes. &lt;/p&gt; &lt;p&gt;  Elle est également active dans la promotion de la diversité en philosophie et a cofondé le "Women in Philosophy Task Force" au Royaume-Uni pour lutter contre le sexisme dans le milieu académique. &lt;/p&gt; &lt;p&gt;  Elle intervient régulièrement dans des  &lt;a href="https://www.youtube.com/watch?v=QDcuCIqCWdQ&amp;t=13s" style="color:#88A1E9" title=" Interview: Jenny Saul and Nadia Mehdi par The Royal Institute of Philosophy"&gt;débats publics&lt;/a&gt; sur le harcèlement, les inégalités de genre et les politiques universitaires. Elle combine une méthodologie analytique avec une perspective clairement engagée, montrant comment la philosophie peut éclairer des problèmes sociaux urgents. Son travail est influent aussi bien en philosophie académique que dans les discussions sur les politiques publiques. &lt;/p&gt; </t>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Jennifer_Saul" title=" Wikipedia"&gt;Jennifer SAUL&lt;/a&gt;  est une philosophe américaine  spécialisée en philosophie du langage, en philosophie féministe et en philosophie de l'esprit. Elle est connue pour ses travaux sur les &lt;a href="https://www.youtube.com/watch?v=2_FqrHs9S-s" title="Jennifer Saul: 'Why Implicit Bias Matters' par The Royal Institute of Philosophy"&gt;biais implicites&lt;/a&gt; et de leur impact sur les comportements sociaux. Elle explore comment ils influencent les décisions, les interactions et les structures sociales, même en l'absence de préjugés explicites, le langage et le genre, ainsi que pour ses analyses des questions liées à la discrimination et à l'oppression. &lt;/p&gt; &lt;p&gt; Elle s'intéresse aussi à la manière dont le langage peut véhiculer des stéréotypes et renforcer des inégalités, même lorsque les locuteurs n'en ont pas conscience. Son livre "Lying, Misleading, and What Is Said" aborde notamment les questions de tromperie et de manipulation linguistique. &lt;/p&gt; &lt;p&gt; Dans son ouvrage  "Feminism: Issues &amp; Arguments", elle examine des débats clés du féminisme, comme la définition du genre, l'objectification ou les controverses autour de la pornographie et de la prostitution. Elle défend une approche analytique rigoureuse des questions féministes. &lt;/p&gt; &lt;p&gt;  Elle est également active dans la promotion de la diversité en philosophie et a cofondé le "Women in Philosophy Task Force" au Royaume-Uni pour lutter contre le sexisme dans le milieu académique. &lt;/p&gt; &lt;p&gt;  Elle intervient régulièrement dans des  &lt;a href="</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">https://www.youtube.com/watch?v=QDcuCIqCWdQ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" s title=" Interview: Jenny Saul and Nadia Mehdi par The Royal Institute of Philosophy"&gt;débats publics&lt;/a&gt; sur le harcèlement, les inégalités de genre et les politiques universitaires. Elle combine une méthodologie analytique avec une perspective clairement engagée, montrant comment la philosophie peut éclairer des problèmes sociaux urgents. Son travail est influent aussi bien en philosophie académique que dans les discussions sur les politiques publiques. &lt;/p&gt; </t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">QZUDokfLdAU</t>
@@ -2288,7 +2315,13 @@
     <t xml:space="preserve">https://www.laphilo.fr/pho/saul-mini.webp</t>
   </si>
   <si>
-    <t xml:space="preserve">philosophe britannique connue pour ses travaux sur les biais implicites, le langage et le genre.</t>
+    <t xml:space="preserve">langage ; ethique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analytique ; Féminisme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">philosophe américaine connue pour ses travaux sur les biais implicites, le langage et le genre.</t>
   </si>
   <si>
     <t xml:space="preserve">Timothy MORTON</t>
@@ -2510,9 +2543,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.laphilo.fr/pho/jenkins-mini.webp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analytique ; Féminisme</t>
   </si>
   <si>
     <t xml:space="preserve">philosophe canadienne connue pour ses travaux sur la métaphysique, l’épistémologie et la philosophie de l’amour. </t>
@@ -2700,7 +2730,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2825,6 +2855,13 @@
       <sz val="9"/>
       <name val="Microsoft YaHei"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -6399,7 +6436,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="177.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="224.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="n">
         <v>1966</v>
       </c>
@@ -6436,7 +6473,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="196.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="n">
         <v>1968</v>
       </c>
@@ -6464,13 +6501,13 @@
         <v>51</v>
       </c>
       <c r="K88" s="2" t="s">
-        <v>88</v>
+        <v>662</v>
       </c>
       <c r="L88" s="2" t="s">
-        <v>53</v>
+        <v>663</v>
       </c>
       <c r="M88" s="2" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="201" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6482,19 +6519,19 @@
         <v>656</v>
       </c>
       <c r="D89" s="8" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="F89" s="7" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="G89" s="10" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="H89" s="10" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="I89" s="10"/>
       <c r="J89" s="1" t="s">
@@ -6504,10 +6541,10 @@
         <v>259</v>
       </c>
       <c r="L89" s="2" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="M89" s="2" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6519,19 +6556,19 @@
         <v>656</v>
       </c>
       <c r="D90" s="8" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="E90" s="12" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="F90" s="7" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="G90" s="10" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="H90" s="10" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="I90" s="10"/>
       <c r="J90" s="1" t="s">
@@ -6541,10 +6578,10 @@
         <v>327</v>
       </c>
       <c r="L90" s="2" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="M90" s="2" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6556,19 +6593,19 @@
         <v>1968</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="E91" s="12" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="F91" s="7" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="G91" s="10" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="H91" s="12" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="I91" s="10"/>
       <c r="J91" s="1" t="s">
@@ -6581,7 +6618,7 @@
         <v>654</v>
       </c>
       <c r="M91" s="2" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="110.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6590,22 +6627,22 @@
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="D92" s="8" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="E92" s="10" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="F92" s="7" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="G92" s="10" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="H92" s="10" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="I92" s="10"/>
       <c r="J92" s="1" t="s">
@@ -6618,7 +6655,7 @@
         <v>53</v>
       </c>
       <c r="M92" s="2" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="145.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6627,26 +6664,26 @@
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="D93" s="8" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="F93" s="7" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="G93" s="10" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="H93" s="10" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="I93" s="10"/>
       <c r="J93" s="1" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="K93" s="2" t="s">
         <v>114</v>
@@ -6655,7 +6692,7 @@
         <v>53</v>
       </c>
       <c r="M93" s="2" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6664,22 +6701,22 @@
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="D94" s="8" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="E94" s="9" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="F94" s="7" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="G94" s="10" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H94" s="10" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="I94" s="10"/>
       <c r="J94" s="1" t="s">
@@ -6692,7 +6729,7 @@
         <v>523</v>
       </c>
       <c r="M94" s="2" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="163.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6701,22 +6738,22 @@
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="D95" s="23" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="E95" s="12" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="F95" s="7" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G95" s="10" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="H95" s="10" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="I95" s="10"/>
       <c r="J95" s="1" t="s">
@@ -6726,10 +6763,10 @@
         <v>42</v>
       </c>
       <c r="L95" s="2" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="M95" s="14" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="117.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6738,35 +6775,35 @@
       </c>
       <c r="B96" s="7"/>
       <c r="C96" s="7" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="D96" s="8" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="F96" s="7" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="G96" s="10" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="H96" s="10" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="I96" s="10"/>
       <c r="J96" s="1" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="K96" s="2" t="s">
         <v>502</v>
       </c>
       <c r="L96" s="2" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="M96" s="2" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6775,22 +6812,22 @@
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="D97" s="8" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="E97" s="12" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="F97" s="7" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="G97" s="10" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="H97" s="10" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="I97" s="10"/>
       <c r="J97" s="1" t="s">
@@ -6803,7 +6840,7 @@
         <v>53</v>
       </c>
       <c r="M97" s="2" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="174" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6812,22 +6849,22 @@
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="D98" s="8" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="E98" s="10" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="F98" s="7" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="G98" s="10" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="H98" s="10" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="I98" s="10"/>
       <c r="J98" s="1" t="s">
@@ -6837,10 +6874,10 @@
         <v>313</v>
       </c>
       <c r="L98" s="2" t="s">
-        <v>735</v>
+        <v>663</v>
       </c>
       <c r="M98" s="14" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="222.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6849,22 +6886,22 @@
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="D99" s="8" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="F99" s="7" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="G99" s="10" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="H99" s="10" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="I99" s="10"/>
       <c r="J99" s="1" t="s">
@@ -6874,10 +6911,10 @@
         <v>451</v>
       </c>
       <c r="L99" s="2" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="M99" s="2" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6886,22 +6923,22 @@
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="D100" s="8" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="E100" s="12" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="F100" s="7" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="G100" s="10" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="H100" s="10" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="I100" s="10"/>
       <c r="J100" s="1" t="s">
@@ -6914,7 +6951,7 @@
         <v>638</v>
       </c>
       <c r="M100" s="2" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6923,22 +6960,22 @@
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="D101" s="8" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="E101" s="12" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="F101" s="7" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="G101" s="10" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="H101" s="10" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="I101" s="10"/>
       <c r="J101" s="1" t="s">
@@ -6951,7 +6988,7 @@
         <v>53</v>
       </c>
       <c r="M101" s="2" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6960,26 +6997,26 @@
       </c>
       <c r="B102" s="7"/>
       <c r="C102" s="7" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="D102" s="8" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="E102" s="10" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="F102" s="7" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="G102" s="10" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="H102" s="10" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="I102" s="10"/>
       <c r="J102" s="1" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="K102" s="2" t="s">
         <v>502</v>
@@ -6988,7 +7025,7 @@
         <v>53</v>
       </c>
       <c r="M102" s="2" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="142.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6997,22 +7034,22 @@
       </c>
       <c r="B103" s="7"/>
       <c r="C103" s="7" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="D103" s="8" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="F103" s="7" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="G103" s="10" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="H103" s="10" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="I103" s="10"/>
       <c r="J103" s="1" t="s">
@@ -7025,7 +7062,7 @@
         <v>53</v>
       </c>
       <c r="M103" s="2" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="125.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7034,22 +7071,22 @@
       </c>
       <c r="B104" s="7"/>
       <c r="C104" s="7" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="D104" s="8" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="E104" s="12" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="F104" s="7" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="G104" s="10" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="H104" s="10" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="I104" s="10"/>
       <c r="J104" s="1" t="s">
@@ -7062,7 +7099,7 @@
         <v>53</v>
       </c>
       <c r="M104" s="2" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="138" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7071,22 +7108,22 @@
       </c>
       <c r="B105" s="7"/>
       <c r="C105" s="7" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="D105" s="8" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="F105" s="7" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="G105" s="10" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="H105" s="10" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="I105" s="10"/>
       <c r="J105" s="1" t="s">
@@ -7096,10 +7133,10 @@
         <v>42</v>
       </c>
       <c r="L105" s="2" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="M105" s="2" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7108,22 +7145,22 @@
       </c>
       <c r="B106" s="7"/>
       <c r="C106" s="7" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="D106" s="23" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="E106" s="10" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="F106" s="7" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="G106" s="10" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="H106" s="10" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="I106" s="10"/>
       <c r="J106" s="1" t="s">
@@ -7133,10 +7170,10 @@
         <v>42</v>
       </c>
       <c r="L106" s="2" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="M106" s="2" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -7203,14 +7240,15 @@
     <hyperlink ref="E82" r:id="rId55" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Iain_Hamilton_Grant&quot;  title=&quot; Wikipedia&quot;&gt;Iain HAMILTON GRAND&lt;/a&gt; est un philosophe britanique, maître de conférences et sa pensée est particulièrement influente dans le courant du &lt;a href=&quot;https://fr.wikipedia.org/wiki/R%C3%A9alisme_sp%C3%A9culatif&quot;  title=&quot;speculative realism  par Wikipedia&quot;&gt;réalisme spéculatif&lt;/a&gt;, auquel il apporte une contribution originale par une ontologie centrée sur la nature et le domaine inorganique. Il a écrit sa thèse sur Kant et Lyotard à l’Université de Warwick, où il a participé à des travaux interdisciplinaire sur la culture cybernétique. Sa philosophie puise ses sources dans Platon, Friedrich Schelling, mais aussi Gilles Deleuze, tout en s’opposant à Aristote et Kant, critiquant leur réduction de la réalité à sa seule expressibilité humaine. &lt;/p&gt; &lt;p&gt; Son livre majeur,  &lt;a href=&quot;https://www.youtube.com/watch?v=5LGODQdFaw0&quot;  title=&quot;Schelling’s Philosophy of Nature  par Philosophical Bachelor&quot;&gt;&quot;Philosophies of Nature After Schelling&quot;&lt;/a&gt; paru en 2006, renouvelle l’intérêt contemporain pour la philosophie naturelle et l’idéalisme allemand, notamment chez Schelling. Il plaide pour un retour à la question de l’inorganique et propose une critique radicale du primat de l’humanité dans la philosophie continentale, soulignant la nécessité de repenser la nature comme productrice d’activité et de devenir. Son ouvrage &quot;On an Artificial Earth&quot; développe cette dimension en invitant à « renverser Kant » plutôt que Platon, afin de mieux répondre aux défis de la philosophie moderne et des sciences naturelles. &lt;/p&gt; &lt;/p&gt; Il se distingue par une ontologie de la puissance et du devenir, accordant un rôle central à la productivité de la nature et à ses forces et il s’intéresse à la philosophie de la nature, à la métaphysique du processus, à la science et à la condition transcendantale du réel. Son travail s’inscrit à la croisée de l’idéalisme allemand, du matérialisme spéculatif et d’une conception cosmologique de la philosophie, qui traverse la pensée contemporaine.​ &lt;/p&gt; "/>
     <hyperlink ref="E84" r:id="rId56" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hartmut_Rosa&quot;  title=&quot; Wikipedia&quot;&gt;Hartmut ROSA&lt;/a&gt; est un sociologue et philosophe allemand connu pour sa contribution à la &lt;a href=&quot;https://laviedesidees.fr/Naissance-de-la-theorie-critique#page&quot;  style=&quot;color:#88A1E9&quot;  title=&quot;Naissance de la théorie critique par Collège de France &quot;&gt;théorie critique&lt;/a&gt; et pour ses travaux sur le concept de &quot;résonance&quot; et la théorie de l'accélération sociale. Il s'intéresse particulièrement aux dynamiques qui façonnent nos vies dans la société moderne. Selon lui, l'accélération sociale, c'est-à-dire l'augmentation constante du rythme et de l'intensité de nos activités, a des conséquences profondes sur notre expérience du monde et notre relation aux autres.  &lt;/p&gt; &lt;p&gt;&#10;Sa théorie de &lt;a href=&quot;https://www.youtube.com/watch?v=fMd-6viV6Gc&quot;  title=&quot;concepts raisonnance par Sébastien Daxi &quot;&gt;la résonance&lt;/a&gt; propose un moyen de retrouver un lien plus harmonieux avec notre environnement et les autres individus. La résonance se produit lorsque nous entrons en contact authentique avec le monde qui nous entoure, ce qui crée un sentiment d'attachement et de plénitude. Selon Rosa, la quête de résonance est essentielle pour préserver notre bien-être et notre humanité dans une société marquée par l'accélération et la superficialité. &lt;/p&gt; &lt;p&gt;  Il est l'auteur de plusieurs ouvrages, dont &lt;a href=&quot;https://major-prepa.com/culture-generale/hartmut-rosa-la-tripartition-du-monde-la-resonance/&quot; title=&quot;La résonance par Major-prepa &quot;&gt; &quot;Resonanz - Eine Soziologie der Weltbeziehung&quot;&lt;/a&gt; (Résonance - Une sociologie de la relation au monde)  ainsi que  &quot;Resonanz: A Sociology of Our Relationship to the World&quot;  où il propose une théorie de la résonance comme qualité des relations humaines avec le monde. Dans cette théorie, il explique comment les individus recherchent des relations résonantes, c'est-à-dire des relations qui les stimulent et les enrichissent mutuellement.. &lt;/p&gt; &lt;p&gt;&#10;Il est l'un des sociologues émergents et est reconnu pour son ouverture à l'égard des autres théories et traditions. &lt;/p&gt; &lt;audio controls title=&quot;Hartmut ROSA, philosophe de la résonance par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10467-28.09.2018-ITEMA_21828397-2.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &lt;p&gt; &lt;/p&gt;"/>
     <hyperlink ref="H87" r:id="rId57" display="https://www.laphilo.fr/pho/dbenatar-mini.webp"/>
-    <hyperlink ref="E90" r:id="rId58" display="&lt;p&gt;&lt;a href=&quot;https://en.wikipedia.org/wiki/Graham_Harman&quot;   title=&quot; Wikipedia&quot;&gt;Graham HARMAN&lt;/a&gt; est un philosophe américain, figure clé du mouvement du &lt;a href=&quot;https://www.youtube.com/watch?v=2voNdhpfbm0&amp;t=190s&quot; style=&quot;color:#88A1E9&quot; title=&quot; Speculative Realism | Graham Harman par The Institute of Art and Ideas &quot;&gt;&quot;réalisme spéculatif&quot;&lt;/a&gt; et co-fondateur de l'ontologie orientée objet (OOO). Sa  philosophie est une réaction contre ce qu'il appelle le &quot;corrélationnisme&quot;, l'idée selon laquelle l'existence de la réalité est inséparable de la perception humaine. Il cherche à redonner une  &lt;a href=&quot;https://www.youtube.com/watch?v=KTeyDSDcXzQ&quot;  title=&quot; Des choses dans le vide. Ce qu'on peut apprendre de Graham Harman par Ars Industrialis &quot;&gt; place centrale aux objets&lt;/a&gt;, qu'ils soient réels, fictifs, naturels, artificiels, humains ou non-humains, en affirmant leur existence indépendante de notre esprit et même de leurs relations causales. &lt;/p&gt; &lt;p&gt;  &lt;a href=&quot;https://www.youtube.com/watch?v=uxDmQ-Hn2X0&quot;  title=&quot;  Object-Oriented Ontology: A New Theory of Everything w/ Graham Harman par derek g larson &quot;&gt; (OOO) &lt;/a&gt; est le cœur de sa philosophie. Il affirme que les objets sont les entités fondamentales de la réalité. Chacun d'eux, qu'il s'agisse d'une tasse de café, d'une montagne, d'un État ou d'une idée, possède une existence autonome et &quot;se retire&quot; de la pleine compréhension, que ce soit par un esprit humain ou par d'autres objets. Pour lui les objets ne peuvent jamais être pleinement appréhendés ou épuisés par nos sens, notre intellect ou même par leurs interactions avec d'autres objets. Il y a toujours une part de l'objet qui reste cachée, insaisissable, une &quot;réalité souterraine&quot; des choses. &lt;/p&gt; &lt;p&gt; Il distingue les objets réels, qui existent indépendamment de toute perception, des objets sensuels, qui sont les objets tels qu'ils nous apparaissent ou tels qu'ils interagissent avec d'autres objets. La tension entre ce que l'objet est réellement (son retrait) et ce qu'il nous présente ou ce qu'il est pour d'autres objets est une dynamique importante de sa pensée. &lt;/p&gt; &lt;p&gt; Il  privilégient l'épistémologie ou l'éthique et met l'accent sur la métaphysique (l'étude de la nature de la réalité). Il considère également que &lt;a href=&quot;https://www.youtube.com/watch?v=QJ0GR9bf00g&quot; title=&quot; Graham Harman: Objects and the Arts par ICA &quot;&gt; l'esthétique &lt;/a&gt; joue un rôle fondamental dans notre appréhension des objets, car l'art, la littérature et la métaphore peuvent nous donner un accès indirect à la réalité retirée des objets, là où la connaissance conceptuelle échoue. &lt;/p&gt; "/>
-    <hyperlink ref="H91" r:id="rId59" display="https://www.laphilo.fr/pho/tgiraud-mini.webp"/>
-    <hyperlink ref="E94" r:id="rId60" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Alexander_Schnell&quot; title=&quot; Wikipedia&quot;&gt;Alexander SCHNELL&lt;/a&gt;   est un philosophe  germano-bulgare spécialiste de l'idéalisme allemand (Kant, Fichte, Schelling) et de la phénoménologie (Husserl, Heidegger, Fink, Richir, Lévinas), il publie une trentaine d'ouvrages en français et allemand, comme Husserl et les fondements de la phénoménologie constructive (2007), Was ist Phänomenologie? (2019) ou sa trilogie récente : La déhiscence du sens (2015), Le clignotement de l’être (2021) et Préphénoménalité et générativité (2025). Il traduit aussi des textes philosophiques et édite des volumes collectifs. &lt;/p&gt; &lt;p&gt; Il développe une &lt;a href=&quot;https://www.youtube.com/watch?v=PuQPvr3xhEM&quot; title=&quot;Prephenomenalité alexxander Schnell et Charles Bobant par Salon Tout Art&quot;&gt;« phénoménologie constructive » &lt;/a&gt; ou « transcendantalisme spéculatif », reprenant le projet husserlien d'une phénoménologie de la connaissance comme idéalisme transcendantal, en intégrant imagination, inconscient phénoménologique, préphénoménalité et générativité. Ses travaux lient philosophie allemande classique, phénoménologie allemande et française, avec des accents sur esthétique et anthropologie, critiquant le primat descriptif au profit de constructions spéculatives. &lt;/p&gt; &#10;"/>
-    <hyperlink ref="E95" r:id="rId61" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Felwine_Sarr&quot;  title=&quot; Wikipedia&quot;&gt;Fenwine SARR&lt;/a&gt; est un philosophe, écrivain, économiste et musicien sénégalais, figure majeure de la pensée africaine contemporaine, il occupe actuellement la chaire Anne-Marie Bryan à l’Université Duke aux États-Unis, où il est professeur de philosophie africaine contemporaine et diasporique. &lt;/p&gt; &lt;p&gt; Il  est reconnu pour son essai marquant,  &lt;a href=&quot;https://www.youtube.com/watch?v=gty0PculB7U&quot;  title=&quot;Afrotopia par david Mboussou&quot;&gt;&quot;Afrotopia&quot; &lt;/a&gt;  ou il propose à la jeunesse africaine de s’affranchir des blessures du passé pour redevenir sujet de son destin, imaginer librement l’avenir, et construire un horizon fondé sur ses atouts propres, qui invite à repenser le futur du continent africain hors des modèles imposés, en valorisant une utopie africaine propre. Il est aussi auteur de plusieurs ouvrages, dont  &quot;Dahij, Méditations africaines&quot;  , &quot;Habiter le monde&quot; et &quot;Les lieux qu’habitent mes rêves&quot;. &lt;/p&gt;&lt;p&gt; Il invite à repenser le monde et l'Afrique à partir des perspectives et des expériences africaines, au lieu de modèles hérités de l'extérieur. Son œuvre prône une décolonisation des savoirs, une valorisation des potentiels endormis du continent et une ouverture à de nouvelles utopies portées par l’Afrique elle-même. Il  propose une « éthique du voyage » : être  &lt;a href=&quot;https://www.youtube.com/watch?v=TVXc5KT_Z6Q&quot; title=&quot;Felwine Sarr : Laisser le monde plus habitable que nous l’avons trouvé par AFD&quot;&gt;disponible au monde &lt;/a&gt; , sortir des assignations identitaires, multiplier les rencontres et apprendre de l’inattendu, loin des approches extractivistes ou exotiques. Cela implique une capacité à se laisser transformer par les lieux, les autres, et à regarder le monde depuis sa propre place, pour contribuer à une pluralité des voix et des expériences. &lt;/p&gt; &lt;p&gt; Sa philosophie est une invitation à renouer avec les potentiels créateurs de l’Afrique, à valoriser la multiplicité des regards sur le monde, et à engager un projet collectif pour redéfinir le devenir africain et humain à partir de ses propres ressources. &lt;/p&gt; &lt;p&gt;&lt;/p&gt; &lt;p&gt; &lt;/p&gt; &lt;audio controls title=&quot; Felwine Sarr, habiter poétiquement le monde par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/23356-13.08.2022-ITEMA_23105530-2022C48096E0003-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;"/>
-    <hyperlink ref="E97" r:id="rId62" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Joshua_Knobe&quot;  title=&quot; Wikipedia&quot;&gt;Joshua KNOBE&lt;/a&gt; est un philosophe américain,  figure marquante de la  &lt;a href=&quot;https://www.youtube.com/watch?v=t-2QldptRis&quot; style=&quot;color:#88A1E9&quot; title=&quot; Théorie de l'action et Effet Knobe (Introduction à la Philosophie Expérimentale) par Empeiria&quot;&gt;philosophie expérimentale&lt;/a&gt; . Il est actuellement professeur de sciences cognitives et de philosophie à l'Université de Yale. Son domaine de réflexion principal est l'utilisation de méthodes expérimentales issues des sciences cognitives pour aborder des questions philosophiques traditionnelles. Ses travaux portent sur des sujets variés, notamment : &lt;/p&gt; &lt;p&gt; - &lt;a href=&quot;https://www.youtube.com/watch?v=LqJD_l7wHw4&quot;  title=&quot; What is Theory of Mind? par Closer To Truth&quot;&gt;La philosophie de l'esprit&lt;/a&gt; : En étudiant nos intuitions sur la conscience. &lt;/p&gt; &lt;p&gt; - La théorie de l'action : En examinant comment nous attribuons l'intentionnalité. &lt;/p&gt; &lt;p&gt; - L'éthique et la morale : En analysant nos jugements moraux et nos intuitions face à des dilemmes. &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est la découverte et l'analyse de &lt;a href=&quot;https://www.youtube.com/watch?v=MC2bAYaWDNU&quot; title=&quot; What is the Knobe Effect? par Philosophical Questions&quot;&gt;&quot;l'effet Knobe&quot;&lt;/a&gt;. Cet effet met en lumière une asymétrie dans nos jugements d'intentionnalité basée sur la valence morale des conséquences d'une action. En d'autres termes, nous sommes plus enclins à juger qu'une personne a intentionnellement causé un effet négatif (même si ce n'était pas son but principal) que si elle a causé un effet positif de manière similaire. &lt;/p&gt; &lt;p&gt; Par exemple, dans un scénario classique, un PDG lance un projet qui augmente les profits de son entreprise mais nuit également à l'environnement. La plupart des gens jugent que le PDG a intentionnellement nui à l'environnement. Cependant, dans un scénario où le même projet profite à l'environnement en plus d'augmenter les profits, les gens sont moins enclins à dire que le PDG a intentionnellement aidé l'environnement. &lt;/p&gt; "/>
-    <hyperlink ref="E100" r:id="rId63" display="&lt;p&gt; &lt;a href=&quot;https://fr.wikipedia.org/wiki/Markus_Gabriel&quot;   title=&quot; Wikipedia&quot;&gt; Markus GABRIEL&lt;/a&gt; est un jeune philosophe Allemand qui est une figure de plus en plus remarquée dans le paysage philosophique mondial. Affirmant une rupture radicale avec la pensée occidentale, il prône un  &lt;a href=&quot;https://www.lesinrocks.com/livres/markus-gabriel-existe-excepte-monde-105595-30-09-2014/&quot;   title=&quot;Markus Gabriel par les Inrockuptibles&quot;&gt;“nouveau réalisme”&lt;/a&gt;.  &lt;/p&gt; &lt;p&gt; Il s'est fait connaître pour sa théorie de &lt;a href=&quot;https://fr.wikipedia.org/wiki/Ontologie_(philosophie)&quot;  title=&quot;Ontologie par Wikipédia&quot;&gt;l'ontologie&lt;/a&gt; nouvelle, qui propose une conception nouvelle de la réalité, en opposition à la métaphysique traditionnelle. Selon lui, la réalité n'est pas quelque chose qui existe en soi, indépendamment de notre perception et de notre connaissance, mais plutôt quelque chose qui est créé par notre propre activité cognitive. Autrement dit, la réalité est une construction sociale, qui dépend de notre langage et de notre culture et non de la perception humaine et qui existe indépendamment de notre esprit. &lt;/p&gt; &lt;p&gt; &#10;Il a écrit de nombreux livres, dont  « Pourquoi le monde n'existe pas », « Je ne suis pas un cerveau : philosophie de l'esprit pour le 21e siècle » et  &lt;a href=&quot;https://www.youtube.com/watch?v=cRxd09vFcxg&amp;ab_channel=FRANCE24&quot;     style=&quot;color:#88A1E9&quot;  title=&quot;Le pouvoir de l'Art par France 24&quot;&gt;&quot; Le pouvoir de 'Art&quot;&lt;/a&gt; . &lt;/p&gt; &lt;p&gt; Il contribue également régulièrement à divers journaux et magazines et est apparu dans de nombreuses émissions de télévision et de radio pour discuter de ses idées. &lt;/p&gt;   &lt;audio controls title=&quot;Si google anticipe pour moi, cela ne veut pas dire qu'il choisit pour moi  par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/16602-10.02.2017-ITEMA_21225836-0.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &lt;p&gt; &lt;/p&gt;"/>
-    <hyperlink ref="E101" r:id="rId64" display="&lt;p&gt;&lt;a href=&quot;https://www.robindembroff.com/&quot;  title=&quot; Wikipedia&quot;&gt;Robin DEMBROFF&lt;/a&gt; est un(e) philosophe américaine travaillant sur les questions de genre, ancré dans la métaphysique, la philosophie du genre, et la théorie queer, iel soulève les zones floues de l’identité en interrogant les catégories qui nous définissent, les mots que l’on utilise pour dire &quot;homme&quot;, &quot;femme&quot;, &quot;non-binaire&quot;, et surtout : pourquoi ces mots ont tant de poids sur nos vies. &lt;/p&gt; &lt;p&gt;  Robin se pose une question simple mais explosive : Et si le genre n’était pas ce que l’on croit ? De là naît une série de textes qui dérangent, qui déplacent, qui éclairent. Iel refuse les définitions rigides car le genre est une construction sociale, oui, mais c’est aussi un  &lt;a href=&quot;https://www.youtube.com/watch?v=-mHFFs49S3o&quot; title=&quot;Robin Dembroff presents at the 2022 Gender and Work Symposium par Havard Business School&quot;&gt;champ de bataille&lt;/a&gt;, un territoire politique, et un espace de résistance. Iel y développe l’idée que l’identité non-binaire n’est pas seulement une absence ou un entre-deux du masculin et du féminin, mais une &lt;a href=&quot;https://www.youtube.com/watch?v=-pNmvthQLds&quot;  title=&quot;&#10;What is sexual orientation? Part I par Center for Philosophy of Religion&quot;&gt;position à part entière&lt;/a&gt;. Une manière de dire non au système de genre binaire, tout en affirmant sa propre existence. &lt;/p&gt; &lt;p&gt; Dans ses écrits – parfois techniques, toujours engagés – on sent la chaleur d’un feu ancien : celui de la justice. Iel écrit comme on lutte, avec précision, mais aussi avec une tendresse désarmante pour celles et ceux qui cherchent leur place dans un monde trop étroit. &lt;/p&gt; "/>
-    <hyperlink ref="E104" r:id="rId65" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Amia_Srinivasan&quot;  title=&quot; Wikipedia&quot;&gt;Amia SRINIVASAN&lt;/a&gt; est une femme philosophe d'origine indienne qui a grandi entre Taïwan, Singapour, New York et Londres. Son parcours cosmopolite a nourri une pensée profondément ancrée dans les réalités multiples du monde contemporain. &lt;/p&gt; &lt;p&gt;  En janvier 2020, elle devient la première femme et la première personne de couleur à occuper la prestigieuse chaire Chichele de théorie sociale et politique à l'université d'Oxford. Son travail se concentre sur l'épistémologie, la philosophie politique, la métaphilosophie et la &lt;a href=&quot;https://www.lesinrocks.com/livres/amia-srinivasan-une-nouvelle-voix-feministe-503329-05-10-2022/&quot; title=&quot;THE RIGHT TO SEX | Amia Srinivasan &amp; Sarah Leonard par Books Are Magic&quot;&gt;théorie féministe&lt;/a&gt; . &lt;/p&gt; &lt;p&gt; Son ouvrage majeur, &lt;a href=&quot;https://www.youtube.com/watch?v=6NjzLlQG5cU&quot;   title=&quot;Amia Srinivasan, une nouvelle voix féministe par Les Inrockuptibles&quot;&gt;Le droit au sexe&lt;/a&gt;, publié en 2021, est une collection d'essais qui explore les intersections entre le désir sexuel, le pouvoir, la race et le genre. Elle y examine comment les normes sociales et politiques influencent nos désirs et comportements sexuels, abordant des sujets tels que le racisme sexuel, les incels, le capitalisme et le mouvement #MeToo.  Elle a aussi publié des articles dans des revues prestigieuses telles que The Philosophical Review, Journal of Political Philosophy et Philosophy &amp; Phenomenological Research. Elle est également éditrice contributrice pour la London Review of Books. &lt;/p&gt; &lt;p&gt; Actuellement, elle travaille sur un second livre intitulé &quot;The Contingent World: Genealogy, Epistemology, Politics&quot;, qui portera sur la pratique de la généalogie critique. Elle s'intéresse également à la place des mouvements identitaires dans la gauche politique, à la philosophie de l'histoire et aux droits des animaux. &lt;/p&gt;"/>
+    <hyperlink ref="E88" r:id="rId58" display="https://www.youtube.com/watch?v=QDcuCIqCWdQ"/>
+    <hyperlink ref="E90" r:id="rId59" display="&lt;p&gt;&lt;a href=&quot;https://en.wikipedia.org/wiki/Graham_Harman&quot;   title=&quot; Wikipedia&quot;&gt;Graham HARMAN&lt;/a&gt; est un philosophe américain, figure clé du mouvement du &lt;a href=&quot;https://www.youtube.com/watch?v=2voNdhpfbm0&amp;t=190s&quot; style=&quot;color:#88A1E9&quot; title=&quot; Speculative Realism | Graham Harman par The Institute of Art and Ideas &quot;&gt;&quot;réalisme spéculatif&quot;&lt;/a&gt; et co-fondateur de l'ontologie orientée objet (OOO). Sa  philosophie est une réaction contre ce qu'il appelle le &quot;corrélationnisme&quot;, l'idée selon laquelle l'existence de la réalité est inséparable de la perception humaine. Il cherche à redonner une  &lt;a href=&quot;https://www.youtube.com/watch?v=KTeyDSDcXzQ&quot;  title=&quot; Des choses dans le vide. Ce qu'on peut apprendre de Graham Harman par Ars Industrialis &quot;&gt; place centrale aux objets&lt;/a&gt;, qu'ils soient réels, fictifs, naturels, artificiels, humains ou non-humains, en affirmant leur existence indépendante de notre esprit et même de leurs relations causales. &lt;/p&gt; &lt;p&gt;  &lt;a href=&quot;https://www.youtube.com/watch?v=uxDmQ-Hn2X0&quot;  title=&quot;  Object-Oriented Ontology: A New Theory of Everything w/ Graham Harman par derek g larson &quot;&gt; (OOO) &lt;/a&gt; est le cœur de sa philosophie. Il affirme que les objets sont les entités fondamentales de la réalité. Chacun d'eux, qu'il s'agisse d'une tasse de café, d'une montagne, d'un État ou d'une idée, possède une existence autonome et &quot;se retire&quot; de la pleine compréhension, que ce soit par un esprit humain ou par d'autres objets. Pour lui les objets ne peuvent jamais être pleinement appréhendés ou épuisés par nos sens, notre intellect ou même par leurs interactions avec d'autres objets. Il y a toujours une part de l'objet qui reste cachée, insaisissable, une &quot;réalité souterraine&quot; des choses. &lt;/p&gt; &lt;p&gt; Il distingue les objets réels, qui existent indépendamment de toute perception, des objets sensuels, qui sont les objets tels qu'ils nous apparaissent ou tels qu'ils interagissent avec d'autres objets. La tension entre ce que l'objet est réellement (son retrait) et ce qu'il nous présente ou ce qu'il est pour d'autres objets est une dynamique importante de sa pensée. &lt;/p&gt; &lt;p&gt; Il  privilégient l'épistémologie ou l'éthique et met l'accent sur la métaphysique (l'étude de la nature de la réalité). Il considère également que &lt;a href=&quot;https://www.youtube.com/watch?v=QJ0GR9bf00g&quot; title=&quot; Graham Harman: Objects and the Arts par ICA &quot;&gt; l'esthétique &lt;/a&gt; joue un rôle fondamental dans notre appréhension des objets, car l'art, la littérature et la métaphore peuvent nous donner un accès indirect à la réalité retirée des objets, là où la connaissance conceptuelle échoue. &lt;/p&gt; "/>
+    <hyperlink ref="H91" r:id="rId60" display="https://www.laphilo.fr/pho/tgiraud-mini.webp"/>
+    <hyperlink ref="E94" r:id="rId61" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Alexander_Schnell&quot; title=&quot; Wikipedia&quot;&gt;Alexander SCHNELL&lt;/a&gt;   est un philosophe  germano-bulgare spécialiste de l'idéalisme allemand (Kant, Fichte, Schelling) et de la phénoménologie (Husserl, Heidegger, Fink, Richir, Lévinas), il publie une trentaine d'ouvrages en français et allemand, comme Husserl et les fondements de la phénoménologie constructive (2007), Was ist Phänomenologie? (2019) ou sa trilogie récente : La déhiscence du sens (2015), Le clignotement de l’être (2021) et Préphénoménalité et générativité (2025). Il traduit aussi des textes philosophiques et édite des volumes collectifs. &lt;/p&gt; &lt;p&gt; Il développe une &lt;a href=&quot;https://www.youtube.com/watch?v=PuQPvr3xhEM&quot; title=&quot;Prephenomenalité alexxander Schnell et Charles Bobant par Salon Tout Art&quot;&gt;« phénoménologie constructive » &lt;/a&gt; ou « transcendantalisme spéculatif », reprenant le projet husserlien d'une phénoménologie de la connaissance comme idéalisme transcendantal, en intégrant imagination, inconscient phénoménologique, préphénoménalité et générativité. Ses travaux lient philosophie allemande classique, phénoménologie allemande et française, avec des accents sur esthétique et anthropologie, critiquant le primat descriptif au profit de constructions spéculatives. &lt;/p&gt; &#10;"/>
+    <hyperlink ref="E95" r:id="rId62" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Felwine_Sarr&quot;  title=&quot; Wikipedia&quot;&gt;Fenwine SARR&lt;/a&gt; est un philosophe, écrivain, économiste et musicien sénégalais, figure majeure de la pensée africaine contemporaine, il occupe actuellement la chaire Anne-Marie Bryan à l’Université Duke aux États-Unis, où il est professeur de philosophie africaine contemporaine et diasporique. &lt;/p&gt; &lt;p&gt; Il  est reconnu pour son essai marquant,  &lt;a href=&quot;https://www.youtube.com/watch?v=gty0PculB7U&quot;  title=&quot;Afrotopia par david Mboussou&quot;&gt;&quot;Afrotopia&quot; &lt;/a&gt;  ou il propose à la jeunesse africaine de s’affranchir des blessures du passé pour redevenir sujet de son destin, imaginer librement l’avenir, et construire un horizon fondé sur ses atouts propres, qui invite à repenser le futur du continent africain hors des modèles imposés, en valorisant une utopie africaine propre. Il est aussi auteur de plusieurs ouvrages, dont  &quot;Dahij, Méditations africaines&quot;  , &quot;Habiter le monde&quot; et &quot;Les lieux qu’habitent mes rêves&quot;. &lt;/p&gt;&lt;p&gt; Il invite à repenser le monde et l'Afrique à partir des perspectives et des expériences africaines, au lieu de modèles hérités de l'extérieur. Son œuvre prône une décolonisation des savoirs, une valorisation des potentiels endormis du continent et une ouverture à de nouvelles utopies portées par l’Afrique elle-même. Il  propose une « éthique du voyage » : être  &lt;a href=&quot;https://www.youtube.com/watch?v=TVXc5KT_Z6Q&quot; title=&quot;Felwine Sarr : Laisser le monde plus habitable que nous l’avons trouvé par AFD&quot;&gt;disponible au monde &lt;/a&gt; , sortir des assignations identitaires, multiplier les rencontres et apprendre de l’inattendu, loin des approches extractivistes ou exotiques. Cela implique une capacité à se laisser transformer par les lieux, les autres, et à regarder le monde depuis sa propre place, pour contribuer à une pluralité des voix et des expériences. &lt;/p&gt; &lt;p&gt; Sa philosophie est une invitation à renouer avec les potentiels créateurs de l’Afrique, à valoriser la multiplicité des regards sur le monde, et à engager un projet collectif pour redéfinir le devenir africain et humain à partir de ses propres ressources. &lt;/p&gt; &lt;p&gt;&lt;/p&gt; &lt;p&gt; &lt;/p&gt; &lt;audio controls title=&quot; Felwine Sarr, habiter poétiquement le monde par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/23356-13.08.2022-ITEMA_23105530-2022C48096E0003-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;"/>
+    <hyperlink ref="E97" r:id="rId63" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Joshua_Knobe&quot;  title=&quot; Wikipedia&quot;&gt;Joshua KNOBE&lt;/a&gt; est un philosophe américain,  figure marquante de la  &lt;a href=&quot;https://www.youtube.com/watch?v=t-2QldptRis&quot; style=&quot;color:#88A1E9&quot; title=&quot; Théorie de l'action et Effet Knobe (Introduction à la Philosophie Expérimentale) par Empeiria&quot;&gt;philosophie expérimentale&lt;/a&gt; . Il est actuellement professeur de sciences cognitives et de philosophie à l'Université de Yale. Son domaine de réflexion principal est l'utilisation de méthodes expérimentales issues des sciences cognitives pour aborder des questions philosophiques traditionnelles. Ses travaux portent sur des sujets variés, notamment : &lt;/p&gt; &lt;p&gt; - &lt;a href=&quot;https://www.youtube.com/watch?v=LqJD_l7wHw4&quot;  title=&quot; What is Theory of Mind? par Closer To Truth&quot;&gt;La philosophie de l'esprit&lt;/a&gt; : En étudiant nos intuitions sur la conscience. &lt;/p&gt; &lt;p&gt; - La théorie de l'action : En examinant comment nous attribuons l'intentionnalité. &lt;/p&gt; &lt;p&gt; - L'éthique et la morale : En analysant nos jugements moraux et nos intuitions face à des dilemmes. &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est la découverte et l'analyse de &lt;a href=&quot;https://www.youtube.com/watch?v=MC2bAYaWDNU&quot; title=&quot; What is the Knobe Effect? par Philosophical Questions&quot;&gt;&quot;l'effet Knobe&quot;&lt;/a&gt;. Cet effet met en lumière une asymétrie dans nos jugements d'intentionnalité basée sur la valence morale des conséquences d'une action. En d'autres termes, nous sommes plus enclins à juger qu'une personne a intentionnellement causé un effet négatif (même si ce n'était pas son but principal) que si elle a causé un effet positif de manière similaire. &lt;/p&gt; &lt;p&gt; Par exemple, dans un scénario classique, un PDG lance un projet qui augmente les profits de son entreprise mais nuit également à l'environnement. La plupart des gens jugent que le PDG a intentionnellement nui à l'environnement. Cependant, dans un scénario où le même projet profite à l'environnement en plus d'augmenter les profits, les gens sont moins enclins à dire que le PDG a intentionnellement aidé l'environnement. &lt;/p&gt; "/>
+    <hyperlink ref="E100" r:id="rId64" display="&lt;p&gt; &lt;a href=&quot;https://fr.wikipedia.org/wiki/Markus_Gabriel&quot;   title=&quot; Wikipedia&quot;&gt; Markus GABRIEL&lt;/a&gt; est un jeune philosophe Allemand qui est une figure de plus en plus remarquée dans le paysage philosophique mondial. Affirmant une rupture radicale avec la pensée occidentale, il prône un  &lt;a href=&quot;https://www.lesinrocks.com/livres/markus-gabriel-existe-excepte-monde-105595-30-09-2014/&quot;   title=&quot;Markus Gabriel par les Inrockuptibles&quot;&gt;“nouveau réalisme”&lt;/a&gt;.  &lt;/p&gt; &lt;p&gt; Il s'est fait connaître pour sa théorie de &lt;a href=&quot;https://fr.wikipedia.org/wiki/Ontologie_(philosophie)&quot;  title=&quot;Ontologie par Wikipédia&quot;&gt;l'ontologie&lt;/a&gt; nouvelle, qui propose une conception nouvelle de la réalité, en opposition à la métaphysique traditionnelle. Selon lui, la réalité n'est pas quelque chose qui existe en soi, indépendamment de notre perception et de notre connaissance, mais plutôt quelque chose qui est créé par notre propre activité cognitive. Autrement dit, la réalité est une construction sociale, qui dépend de notre langage et de notre culture et non de la perception humaine et qui existe indépendamment de notre esprit. &lt;/p&gt; &lt;p&gt; &#10;Il a écrit de nombreux livres, dont  « Pourquoi le monde n'existe pas », « Je ne suis pas un cerveau : philosophie de l'esprit pour le 21e siècle » et  &lt;a href=&quot;https://www.youtube.com/watch?v=cRxd09vFcxg&amp;ab_channel=FRANCE24&quot;     style=&quot;color:#88A1E9&quot;  title=&quot;Le pouvoir de l'Art par France 24&quot;&gt;&quot; Le pouvoir de 'Art&quot;&lt;/a&gt; . &lt;/p&gt; &lt;p&gt; Il contribue également régulièrement à divers journaux et magazines et est apparu dans de nombreuses émissions de télévision et de radio pour discuter de ses idées. &lt;/p&gt;   &lt;audio controls title=&quot;Si google anticipe pour moi, cela ne veut pas dire qu'il choisit pour moi  par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/16602-10.02.2017-ITEMA_21225836-0.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &lt;p&gt; &lt;/p&gt;"/>
+    <hyperlink ref="E101" r:id="rId65" display="&lt;p&gt;&lt;a href=&quot;https://www.robindembroff.com/&quot;  title=&quot; Wikipedia&quot;&gt;Robin DEMBROFF&lt;/a&gt; est un(e) philosophe américaine travaillant sur les questions de genre, ancré dans la métaphysique, la philosophie du genre, et la théorie queer, iel soulève les zones floues de l’identité en interrogant les catégories qui nous définissent, les mots que l’on utilise pour dire &quot;homme&quot;, &quot;femme&quot;, &quot;non-binaire&quot;, et surtout : pourquoi ces mots ont tant de poids sur nos vies. &lt;/p&gt; &lt;p&gt;  Robin se pose une question simple mais explosive : Et si le genre n’était pas ce que l’on croit ? De là naît une série de textes qui dérangent, qui déplacent, qui éclairent. Iel refuse les définitions rigides car le genre est une construction sociale, oui, mais c’est aussi un  &lt;a href=&quot;https://www.youtube.com/watch?v=-mHFFs49S3o&quot; title=&quot;Robin Dembroff presents at the 2022 Gender and Work Symposium par Havard Business School&quot;&gt;champ de bataille&lt;/a&gt;, un territoire politique, et un espace de résistance. Iel y développe l’idée que l’identité non-binaire n’est pas seulement une absence ou un entre-deux du masculin et du féminin, mais une &lt;a href=&quot;https://www.youtube.com/watch?v=-pNmvthQLds&quot;  title=&quot;&#10;What is sexual orientation? Part I par Center for Philosophy of Religion&quot;&gt;position à part entière&lt;/a&gt;. Une manière de dire non au système de genre binaire, tout en affirmant sa propre existence. &lt;/p&gt; &lt;p&gt; Dans ses écrits – parfois techniques, toujours engagés – on sent la chaleur d’un feu ancien : celui de la justice. Iel écrit comme on lutte, avec précision, mais aussi avec une tendresse désarmante pour celles et ceux qui cherchent leur place dans un monde trop étroit. &lt;/p&gt; "/>
+    <hyperlink ref="E104" r:id="rId66" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Amia_Srinivasan&quot;  title=&quot; Wikipedia&quot;&gt;Amia SRINIVASAN&lt;/a&gt; est une femme philosophe d'origine indienne qui a grandi entre Taïwan, Singapour, New York et Londres. Son parcours cosmopolite a nourri une pensée profondément ancrée dans les réalités multiples du monde contemporain. &lt;/p&gt; &lt;p&gt;  En janvier 2020, elle devient la première femme et la première personne de couleur à occuper la prestigieuse chaire Chichele de théorie sociale et politique à l'université d'Oxford. Son travail se concentre sur l'épistémologie, la philosophie politique, la métaphilosophie et la &lt;a href=&quot;https://www.lesinrocks.com/livres/amia-srinivasan-une-nouvelle-voix-feministe-503329-05-10-2022/&quot; title=&quot;THE RIGHT TO SEX | Amia Srinivasan &amp; Sarah Leonard par Books Are Magic&quot;&gt;théorie féministe&lt;/a&gt; . &lt;/p&gt; &lt;p&gt; Son ouvrage majeur, &lt;a href=&quot;https://www.youtube.com/watch?v=6NjzLlQG5cU&quot;   title=&quot;Amia Srinivasan, une nouvelle voix féministe par Les Inrockuptibles&quot;&gt;Le droit au sexe&lt;/a&gt;, publié en 2021, est une collection d'essais qui explore les intersections entre le désir sexuel, le pouvoir, la race et le genre. Elle y examine comment les normes sociales et politiques influencent nos désirs et comportements sexuels, abordant des sujets tels que le racisme sexuel, les incels, le capitalisme et le mouvement #MeToo.  Elle a aussi publié des articles dans des revues prestigieuses telles que The Philosophical Review, Journal of Political Philosophy et Philosophy &amp; Phenomenological Research. Elle est également éditrice contributrice pour la London Review of Books. &lt;/p&gt; &lt;p&gt; Actuellement, elle travaille sur un second livre intitulé &quot;The Contingent World: Genealogy, Epistemology, Politics&quot;, qui portera sur la pratique de la généalogie critique. Elle s'intéresse également à la place des mouvements identitaires dans la gauche politique, à la philosophie de l'histoire et aux droits des animaux. &lt;/p&gt;"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
31 fiches islam / judaïsme, courants « Philosophie juive médiévale » et « Nahda »
28 fiches dans orientaux, 3 vivants dans autre-actif, médias du Proche-Orient
ancien, bouton « Plan du site » retiré de l'en-tête de l'accueil.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-autre-actif.xlsx
+++ b/data/frise-philosophes-autre-actif.xlsx
@@ -7743,6 +7743,146 @@
         <v>2</v>
       </c>
     </row>
+    <row r="108" customFormat="false" ht="178.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A108" s="7">
+        <v>1933</v>
+      </c>
+      <c r="C108" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1933</t>
+        </is>
+      </c>
+      <c r="D108" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seyyed Hossein NASR</t>
+        </is>
+      </c>
+      <c r="E108" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Seyyed_Hossein_Nasr"  title=" Wikipedia"&gt;Seyyed Hossein NASR&lt;/a&gt; est un philosophe iranien né à Téhéran en 1933. Envoyé aux États-Unis à douze ans, il étudie la physique au MIT, puis l'histoire des sciences à Harvard, où il obtient son doctorat en 1958. Il rentre alors en Iran, enseigne à l'université de Téhéran et fonde en 1974 l'Académie impériale iranienne de philosophie. La révolution de 1979 le contraint à l'exil : il enseigne depuis 1984 à l'université George Washington.&lt;/p&gt; &lt;p&gt;Dès ses études, il est déçu par une science moderne qui ne dit rien du sens des choses, et découvre les auteurs de l'école dite « traditionaliste », René Guénon et Frithjof Schuon. Avec eux, il affirme qu'il existe une sagesse éternelle, la &lt;em&gt;philosophia perennis&lt;/em&gt;, présente au cœur de toutes les grandes religions, et que le monde moderne l'a oubliée.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Connaissance et le Sacré&lt;/em&gt;, issu de conférences prononcées en 1981, il défend l'idée d'une « science sacrée » : connaître vraiment, c'est relier chaque chose à son origine divine. Il a consacré de nombreux ouvrages aux sciences et à la philosophie du monde musulman, d'Avicenne à Molla Sadra, ainsi qu'au soufisme, qu'il pratique lui-même. Il a aussi dirigé une traduction commentée du Coran en anglais, &lt;em&gt;The Study Quran&lt;/em&gt; (2015), qui rassemble les interprétations des différentes écoles.&lt;/p&gt; &lt;p&gt;Dès 1968, dans &lt;em&gt;L'Homme et la Nature&lt;/em&gt;, il soutient que la crise écologique est d'abord une crise spirituelle : en cessant de voir la nature comme sacrée, l'homme moderne s'est cru autorisé à la dominer sans limite. Il est l'un des premiers penseurs à avoir posé ce diagnostic.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J108" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perse</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique ; spiritualite</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pérennialisme ; Soufisme</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe iranien, penseur de la science sacrée et de la tradition, professeur aux États-Unis.</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="178.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="7">
+        <v>1933</v>
+      </c>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1933</t>
+        </is>
+      </c>
+      <c r="D109" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abdallah LAROUI</t>
+        </is>
+      </c>
+      <c r="E109" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Abdallah_Laroui"  title=" Wikipedia"&gt;Abdallah LAROUI&lt;/a&gt; est un historien, philosophe et romancier marocain né à Azemmour en 1933. Après des études à Rabat et à Paris, il enseigne l'histoire à l'université Mohammed V de Rabat pendant plus de trente ans. Il écrit en français et en arabe, et a traduit en arabe des textes de Rousseau et de Montesquieu. Il est aussi l'auteur d'une &lt;em&gt;Histoire du Maghreb&lt;/em&gt; (1970) et de plusieurs romans.&lt;/p&gt; &lt;p&gt;Son premier livre, &lt;em&gt;L'Idéologie arabe contemporaine&lt;/em&gt; (1967), paraît l'année de la défaite arabe face à Israël et devient une référence. Il y décrit trois figures qui, depuis un siècle, répondent chacune à sa façon au défi de l'Occident : le clerc, qui cherche le salut dans le retour à la religion ; le politicien libéral, qui l'attend de la démocratie ; le technophile, qui ne croit qu'à la science et à l'industrie. Aucune, selon lui, ne pense vraiment la situation.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Crise des intellectuels arabes&lt;/em&gt; (1974), il oppose deux attitudes : le traditionalisme, qui cherche dans le passé des réponses toutes faites, et l'historicisme, qu'il défend. Être historiciste, c'est admettre que l'histoire a un sens, que la modernité née en Europe est un acquis de toute l'humanité, et qu'un peuple en retard doit en assimiler les principes : raison, liberté, État, sans croire pouvoir s'en dispenser. Le marxisme l'intéresse surtout comme le résumé de cette pensée moderne.&lt;/p&gt; &lt;p&gt;Il plaide ainsi pour une rupture nette avec l'héritage, là où son compatriote al-Jabri proposait de le relire. Il a poursuivi ce travail dans une série d'ouvrages en arabe, chacun consacré à un concept : l'idéologie, la liberté, l'État, l'histoire, la raison.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J109" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marocaine</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">politique ; epistemologie</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marxisme</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">historien et philosophe marocain, auteur de L'Idéologie arabe contemporaine.</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="178.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A110" s="7">
+        <v>1945</v>
+      </c>
+      <c r="C110" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1945</t>
+        </is>
+      </c>
+      <c r="D110" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abdolkarim SOROUSH</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Abdolkarim_Soroush"  title=" Wikipedia"&gt;Abdolkarim SOROUSH&lt;/a&gt;, nom de plume de Hossein Haj Faraj Dabbagh, est un philosophe iranien né à Téhéran en 1945. Pharmacien de formation, il étudie à Londres la chimie, puis l'histoire et la philosophie des sciences, où il découvre Karl Popper. Rentré en Iran à la révolution de 1979, il siège au conseil chargé de réorganiser les universités, qu'il quitte en 1983. Il devient dans les années 1990 la principale voix des intellectuels réformateurs.&lt;/p&gt; &lt;p&gt;Sa thèse la plus connue est exposée dans &lt;em&gt;La Contraction et l'expansion théoriques de la charia&lt;/em&gt; (1990). Il y distingue la religion elle-même, d'origine divine, et la connaissance que les hommes en ont. Cette connaissance est humaine, faillible et historique : elle dépend de tout ce que nous savons par ailleurs, en science, en histoire ou en philosophie, et change donc avec les époques. Personne ne peut dès lors prétendre détenir l'interprétation définitive, pas même le clergé.&lt;/p&gt; &lt;p&gt;Il en tire une critique du pouvoir religieux : faire de la religion une idéologie d'État, c'est la figer et la corrompre. Un gouvernement peut être à la fois religieux et démocratique, mais seulement s'il respecte la liberté de croire et les droits de l'homme. Il rejette ainsi le principe iranien du gouvernement du juriste-théologien.&lt;/p&gt; &lt;p&gt;Il a ensuite soutenu que la révélation porte la marque de la personnalité et de l'époque du Prophète. Grand lecteur du poète mystique Rumi, il a été agressé et empêché d'enseigner, puis a quitté l'Iran vers 2000 pour les universités américaines et européennes. Il a reçu le prix Érasme en 2004. Il partagea ce prix avec la sociologue marocaine Fatima Mernissi.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J110" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perse</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">epistemologie ; spiritualite ; politique</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Herméneutique</t>
+        </is>
+      </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe iranien, penseur de la réforme religieuse et de la distinction entre religion et connaissance religieuse.</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
+    </row>
     <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Thèmes des vivants : Justice scindé (nouveau thème Critique sociale & capitalisme), nouveau thème Art & esthétique, Esprit renommé ; liens Aujourd'hui sur /definition/ ; dates d'Histoire des philosophes corrigées ; courants de Kautilya et Duras
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-autre-actif.xlsx
+++ b/data/frise-philosophes-autre-actif.xlsx
@@ -3667,7 +3667,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice</t>
+          <t xml:space="preserve">critique</t>
         </is>
       </c>
     </row>
@@ -3712,7 +3712,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice ; continental</t>
+          <t xml:space="preserve">critique ; continental</t>
         </is>
       </c>
     </row>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t xml:space="preserve">continental</t>
+          <t xml:space="preserve">continental ; art</t>
         </is>
       </c>
     </row>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice ; genre</t>
+          <t xml:space="preserve">critique ; genre</t>
         </is>
       </c>
     </row>
@@ -4456,7 +4456,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t xml:space="preserve">reel</t>
+          <t xml:space="preserve">reel ; art</t>
         </is>
       </c>
     </row>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice ; continental</t>
+          <t xml:space="preserve">critique ; continental</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice</t>
+          <t xml:space="preserve">critique</t>
         </is>
       </c>
     </row>
@@ -4774,7 +4774,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t xml:space="preserve">continental</t>
+          <t xml:space="preserve">art</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice ; continental</t>
+          <t xml:space="preserve">critique ; continental</t>
         </is>
       </c>
     </row>
@@ -5005,7 +5005,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice ; genre</t>
+          <t xml:space="preserve">critique ; genre</t>
         </is>
       </c>
     </row>
@@ -5614,7 +5614,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t xml:space="preserve">continental</t>
+          <t xml:space="preserve">art</t>
         </is>
       </c>
     </row>
@@ -5659,7 +5659,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t xml:space="preserve">sens ; continental</t>
+          <t xml:space="preserve">sens ; continental ; art</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t xml:space="preserve">continental</t>
+          <t xml:space="preserve">art</t>
         </is>
       </c>
     </row>
@@ -5935,7 +5935,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t xml:space="preserve">genre ; justice</t>
+          <t xml:space="preserve">genre ; critique</t>
         </is>
       </c>
     </row>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="Q63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">decolonial ; justice</t>
+          <t xml:space="preserve">decolonial ; critique</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice</t>
+          <t xml:space="preserve">critique</t>
         </is>
       </c>
     </row>
@@ -6116,7 +6116,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice</t>
+          <t xml:space="preserve">critique</t>
         </is>
       </c>
     </row>
@@ -6392,7 +6392,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice</t>
+          <t xml:space="preserve">critique</t>
         </is>
       </c>
     </row>
@@ -6620,7 +6620,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice</t>
+          <t xml:space="preserve">critique</t>
         </is>
       </c>
     </row>
@@ -6713,7 +6713,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t xml:space="preserve">esprit-ia ; justice</t>
+          <t xml:space="preserve">esprit-ia ; critique</t>
         </is>
       </c>
     </row>
@@ -6848,7 +6848,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice</t>
+          <t xml:space="preserve">critique</t>
         </is>
       </c>
     </row>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice</t>
+          <t xml:space="preserve">sens</t>
         </is>
       </c>
     </row>
@@ -7166,7 +7166,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t xml:space="preserve">justice</t>
+          <t xml:space="preserve">sens</t>
         </is>
       </c>
     </row>
@@ -7924,7 +7924,7 @@
       </c>
       <c r="Q107" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">genre ; justice</t>
+          <t xml:space="preserve">genre ; critique</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Afrique (8 fiches) et Asie du Sud-Est (10 fiches) ; cartes « Afrique Subsaharienne » et « Asie du Sud-Est » ; groupe asie-se supprimé ; « Pensée juive » dans le catalogue et la recherche ; portraits Yan Fu, Tan Sitong, Livre de Job
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-autre-actif.xlsx
+++ b/data/frise-philosophes-autre-actif.xlsx
@@ -8044,12 +8044,64 @@
       </c>
     </row>
     <row r="109" customFormat="false" ht="205.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="7">
+        <v>1933</v>
+      </c>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1933</t>
+        </is>
+      </c>
+      <c r="D109" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sulak SIVARAKSA</t>
+        </is>
+      </c>
+      <c r="E109" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Sulak_Sivaraksa" title=" Wikipedia (en)"&gt;Sulak SIVARAKSA&lt;/a&gt; est un intellectuel, écrivain et militant thaïlandais, l’une des grandes figures du bouddhisme engagé. Né à Bangkok dans une famille sino-thaïe aisée, il étudie au pays de Galles, à Lampeter, puis devient avocat à Londres en 1961. De retour en Thaïlande, il dirige la &lt;em&gt;Social Science Review&lt;/em&gt;, qui devient dans les années 1960 la grande revue intellectuelle du pays, et fonde en 1968 une fondation qui soutient de nombreuses associations sociales, écologiques et culturelles.&lt;/p&gt; &lt;p&gt;Bouddhiste laïc, il refuse un bouddhisme réduit aux rituels et au mérite individuel, et parle d’un bouddhisme « avec un petit b », tourné vers la justice et la non-violence plutôt que vers les institutions. Pour lui, les trois poisons de l’enseignement du Bouddha, l’avidité, la haine et l’illusion, ne sont pas seulement des fautes personnelles : ils se sont incarnés dans des structures, la société de consommation, le militarisme et les inégalités. Il critique ainsi un modèle de développement importé d’Occident qui détruit les communautés villageoises, la nature et les cultures locales, et lui oppose une économie de la mesure et du partage.&lt;/p&gt; &lt;p&gt;Il est en 1989 l’un des fondateurs du Réseau international des bouddhistes engagés, placé sous le patronage du dalaï-lama et de Thich Nhat Hanh. Ses critiques du pouvoir lui valent d’être poursuivi à plusieurs reprises pour crime de lèse-majesté, en 1984 puis en 1991, ce qui le contraint à l’exil jusqu’à son acquittement en 1995. La même année, il reçoit le &lt;a href="https://fr.wikipedia.org/wiki/Right_Livelihood_Award" title=" Wikipedia"&gt;prix Nobel alternatif&lt;/a&gt;. Parmi ses livres traduits figure &lt;em&gt;Seeds of Peace&lt;/em&gt; (1992).&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="G109" s="1"/>
+      <c r="H109" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/sivaraksa-mini.webp</t>
+        </is>
+      </c>
       <c r="I109" s="1"/>
-      <c r="K109" s="1"/>
-      <c r="L109" s="1"/>
-      <c r="M109" s="1"/>
-      <c r="Q109" s="1"/>
+      <c r="J109" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thaïlandaise</t>
+        </is>
+      </c>
+      <c r="K109" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique ; politique</t>
+        </is>
+      </c>
+      <c r="L109" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bouddhisme Theravada</t>
+        </is>
+      </c>
+      <c r="M109" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">intellectuel bouddhiste thaïlandais, figure du bouddhisme engagé et critique du développement consumériste.</t>
+        </is>
+      </c>
+      <c r="O109" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inde</t>
+        </is>
+      </c>
+      <c r="P109">
+        <v>2</v>
+      </c>
+      <c r="Q109" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sens ; critique</t>
+        </is>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="178.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="0"/>

</xml_diff>

<commit_message>
Mogobe Ramose (né vers 1945) ; Skovoroda ukrainien (colonne Nationalité dans le fichier des Russes, Ukraine dans Europe du Nord & Centrale)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-autre-actif.xlsx
+++ b/data/frise-philosophes-autre-actif.xlsx
@@ -3299,7 +3299,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD111"/>
+  <dimension ref="A1:XFD112"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -8225,6 +8225,64 @@
       <c r="Q111" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">sens</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="178.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A112" s="0">
+        <v>1945</v>
+      </c>
+      <c r="C112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">né vers 1945</t>
+        </is>
+      </c>
+      <c r="D112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mogobe RAMOSE</t>
+        </is>
+      </c>
+      <c r="E112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Mogobe_Ramose" title=" Wikipedia (en)"&gt;Mogobe RAMOSE&lt;/a&gt; est un philosophe sud-africain, l’un de ceux qui ont fait connaître dans le monde entier la philosophie africaine, et en particulier l’&lt;a href="https://fr.wikipedia.org/wiki/Ubuntu_%28philosophie%29" title=" Wikipedia"&gt;ubuntu&lt;/a&gt;. Sa date de naissance n’est pas connue avec précision. Opposant à l’apartheid, il doit quitter son pays et vit longtemps en exil comme réfugié politique en Belgique, où il soutient en 1983 un doctorat de philosophie à l’université catholique de Louvain ; il étudie aussi les relations internationales à la London School of Economics.&lt;/p&gt; &lt;p&gt;Rentré en Afrique du Sud en 1996, il enseigne à l’université du Venda, puis à l’université d’Afrique du Sud, à Pretoria. Dans &lt;em&gt;African Philosophy through Ubuntu&lt;/em&gt; (1999), il fait de l’ubuntu, « une personne est une personne par les autres personnes », une véritable philosophie et non une simple sagesse populaire. Il décompose le mot : &lt;em&gt;ubu&lt;/em&gt; désigne l’être en général, toujours en mouvement, et &lt;em&gt;ntu&lt;/em&gt; sa manifestation concrète dans les êtres et les personnes. Pour l’ubuntu, l’être est un devenir, et la personne n’existe que dans des relations, avec les vivants, les ancêtres et ceux qui ne sont pas encore nés.&lt;/p&gt; &lt;p&gt;Ramose en tire une pensée de la justice : la colonisation et le racisme ont nié l’humanité commune du colonisateur et du colonisé, et la fin de l’apartheid ne suffit pas tant que la conquête, notamment celle des terres, n’a pas été réparée. Héritier du panafricanisme de &lt;a href="https://fr.wikipedia.org/wiki/Robert_Sobukwe" title=" Wikipedia"&gt;Robert Sobukwe&lt;/a&gt;, il critique l’idée, présente chez Hegel, que l’Afrique serait hors de l’histoire et que la raison appartiendrait à l’Occident, et défend un vrai dialogue entre les philosophies du monde.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/ramose-mini.webp</t>
+        </is>
+      </c>
+      <c r="J112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sud-Africaine</t>
+        </is>
+      </c>
+      <c r="K112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique ; politique</t>
+        </is>
+      </c>
+      <c r="L112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ubuntu ; Philosophie africaine</t>
+        </is>
+      </c>
+      <c r="M112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe sud-africain, grand penseur de l’ubuntu comme philosophie de la justice et de la libération.</t>
+        </is>
+      </c>
+      <c r="O112" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="P112" s="0">
+        <v>2</v>
+      </c>
+      <c r="Q112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">decolonial</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vitesse et accessibilité : podcasts non téléchargés avant le clic (/histoire-des-courants/, /definition/), décalages de mise en page supprimés (recherche, grandes frises), ordre des titres de /frises/, zones tactiles de l'arbre ; liens sans adresse corrigés (Nagasawa, Simone Weil)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-autre-actif.xlsx
+++ b/data/frise-philosophes-autre-actif.xlsx
@@ -7770,8 +7770,10 @@
       <c r="D102" s="8" t="s">
         <v>786</v>
       </c>
-      <c r="E102" s="10" t="s">
-        <v>787</v>
+      <c r="E102" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Yujin_Nagasawa"  title=" Wikipedia"&gt;Yujin NAGASAWA&lt;/a&gt; est un philosophe japonnais, professeur à l'Université de Birmingham au Royaume-Uni, où il occupe la chaire de philosophie de la religion. Il est considéré comme l'une des figures les plus importantes et les plus prolifiques dans les domaines de la  &lt;a href="https://www.youtube.com/watch?v=_JgDLjsGXGY" title=" Yujin Nagasawa - Do Religions Complement or Contradict? par Closer To Truth"&gt;  philosophie de la religion&lt;/a&gt;, la philosophie de l'esprit et la métaphysique analytique. Sa renommée est principalement due à son travail sur deux grands problèmes : le problème du mal et l'existence de Dieu. &lt;/p&gt; &lt;p&gt; Il a apporté une contribution majeure au débat séculaire sur le &lt;a href="https://www.youtube.com/watch?v=hHAZnMW0uXA" title=" The Problem of Evil for Non-Theists with Yujin Nagasawa par Furthering Christendom"&gt;problème du mal&lt;/a&gt;. Le problème traditionnel pose que l'existence d'un Dieu omnipotent, omniscient et omnibienveillant est incompatible avec l'existence de la souffrance et du mal dans le monde. Il a proposé une défense innovante appelée "la défense du Dieu ultime" (Maximal God defence). Au lieu de tenter de justifier pourquoi Dieu permettrait le mal, il remet en question la conception même de Dieu qui sous-tend le problème. Il argue que le Dieu de la tradition athée est un "Dieu modaleirement limité", c'est-à-dire un être qui, bien que très puissant, existe simplement dans un monde possible et y exerce ses pouvoirs. Le véritable Dieu ultime doit être un être "modaleirement immuable", qui existe de la même manière dans tous les mondes possibles. Les propriétés d'un tel être seraient si radicalement différentes de notre compréhension que nous ne pouvons pas affirmer avec certitude que le mal que nous observons est logiquement incompatible avec son existence. En d'autres termes, notre cadre conceptuel est trop limité pour juger de ce qu'un Dieu ultime permettrait ou non. &lt;/p&gt; &lt;p&gt; Dans le domaine de la philosophie de l'esprit, il a développé, avec le philosophe australien David Chalmers, une version du panpsychisme appelée &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9orie_du_double_aspect" style="color:#88A1E9" title=" Théorie du double aspect par Wikipedia"&gt;  "la théorie du double aspect du monisme panprotopsychiste"&lt;/a&gt;. Face au "problème difficile de la conscience" (pourquoi l'activité cérébrale produit-elle une expérience subjective ?), cette théorie propose que la matière physique et la conscience (ou du moins des propriétés protoconscientes) sont deux aspects d'une seule et même réalité fondamentale. C'est une tentative élégante de naturaliser la conscience sans tomber dans le réductionnisme matérialiste ni dans un dualisme substance. &lt;/p&gt; &lt;p&gt; Il a également travaillé sur l'immortalité et la vie après la mort, la notion de perfection divine, et les implications philosophiques de la maladie mentale (comme la schizophrénie et le trouble de la personnalité multiple sur la notion de soi). Il est un penseur de premier plan qui, par ses travaux sur le mal, Dieu et la conscience, pousse les frontières de la philosophie analytique et offre des perspectives nouvelles et stimulantes sur certaines des questions les plus profondes de l'humanité. &lt;/p&gt; &lt;p&gt;  Il est un critique important du "vitalisme", l'idée que la vie biologique doit être préservée à tout prix. Il argue que la qualité de la relation que l'on entretient avec sa propre vie est plus importante que la simple prolongation de l'existence biologique. Cela l'amène à des réflexions profondes sur l'euthanasie, les soins palliatifs et l'accompagnement de la fin de vie, où il privilégie une approche centrée sur le sens que la personne donne à sa vie jusqu'à son terme. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F102" s="7" t="s">
         <v>788</v>

</xml_diff>

<commit_message>
Textes des philosophes, lots 1 à 5 : 49 fiches d'importance 3 et 2 portées à 1 400-1 610 caractères (Nkrumah, Yi Hwang, Épictète, Lao Tseu, Zhu Xi, Plotin, Confucius, Nagarjuna, Mencius, Pythagore, Beauvoir, Avicenne, Al-Kindi, Thalès, Averroès, Vivekananda, Sartre, Héraclite, Tsongkhapa, Tchouang-tseu, Spinoza, Ockham, Gandhi, Locke, Marc Aurèle, Bergson, Kant, Hobbes, Heidegger, Hermias d'Alexandrie, Pierre d'Espagne, Zénon de Kition, Proclus, Hermias de Phénicie, Durkheim, Ulrich de Strasbourg, Berkeley, Euclide de Mégare, Albert le Grand, Kuki, Nishi, Watsuji, Itō Jinsai, Tanabe, Hakuin, Comte, Yi Ik, Akshapada Gautama, Graham Priest) ; liens d'origine conservés, lien YouTube d'Ockham et titres de liens mal fermés réparés, lien du nom d'Hermias de Phénicie corrigé ; vidéo de Moïse de León (éditeur)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-autre-actif.xlsx
+++ b/data/frise-philosophes-autre-actif.xlsx
@@ -4934,8 +4934,10 @@
       <c r="D37" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>297</v>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Graham_Priest" title=" Wikipedia"&gt;Graham Priest&lt;/a&gt; (né en 1948) est un philosophe et logicien britannique installé en Australie, puis aux États-Unis, connu pour défendre une thèse qui semble absurde : certaines contradictions sont vraies. Né à Londres, formé aux mathématiques à Cambridge, il enseigne à l’université de Melbourne, puis à la City University de New York.&lt;/p&gt; &lt;p&gt;Depuis Aristote, le principe de non-contradiction passe pour la loi la plus sûre de la pensée : une proposition et sa négation ne peuvent être vraies ensemble. En logique classique, une seule contradiction permet même de démontrer n’importe quoi. Priest défend au contraire le « dialéthéisme » : il existe des énoncés à la fois vrais et faux. Le meilleur exemple est le &lt;a href="https://fr.wikipedia.org/wiki/Paradoxe_du_menteur" title=" Wikipedia"&gt;paradoxe du menteur&lt;/a&gt; : la phrase « cette phrase est fausse » est fausse si elle est vraie, et vraie si elle est fausse. Plutôt que d’interdire de telles phrases, Priest les accepte comme de vraies contradictions, et construit dès 1979 une « logique du paradoxe », une &lt;a href="https://fr.wikipedia.org/wiki/Logique_paraconsistante" title=" Wikipedia"&gt;logique paraconsistante&lt;/a&gt; dans laquelle une contradiction ne fait pas s’effondrer tout le raisonnement. Il expose cette position dans &lt;em&gt;In Contradiction&lt;/em&gt; (1987). Dans &lt;em&gt;Beyond the Limits of Thought&lt;/em&gt; (1995), il montre que les grands philosophes, de Kant à Hegel et de Wittgenstein à Derrida, rencontrent des contradictions dès qu’ils tentent de penser les limites de la pensée.&lt;/p&gt; &lt;p&gt;Il s’intéresse aussi à la philosophie bouddhiste, en particulier au tétralemme et à la dialectique de &lt;a href="https://fr.wikipedia.org/wiki/N%C4%81g%C4%81rjuna" title=" Wikipedia"&gt;Nagarjuna&lt;/a&gt;, qu’il éclaire avec ses outils logiques, et il défend une théorie des objets qui n’existent pas.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F37" s="1" t="s">
         <v>298</v>

</xml_diff>

<commit_message>
Textes des philosophes, lots 6 à 11 : 60 fiches portées à 1 400-1 620 caractères (de Nguyễn Trãi, Wasil ibn Ata, Gramsci… à Lucrèce, Cassiodore, Markus Gabriel) ; erreurs corrigées (Gabriel, Panétios, Cassiodore, Mani, Pittacos, Thémistios, Onfray, Bède, Aidésia…), liens d'origine conservés, lien Palingénésie de Bonnet replacé, vidéo de Brugère corrigée ; éditeur : Ménissier (lien du blog), vidéo de Fontenelle, portraits de Fontenelle et Moïse de León
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-autre-actif.xlsx
+++ b/data/frise-philosophes-autre-actif.xlsx
@@ -3899,8 +3899,7 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Eb%C3%A9n%C3%A9zer_Njoh-Mouell%C3%A9"  title=" Wikipedia"&gt;Ebénézer NJOH-MOUELLÉ&lt;/a&gt;  est un philosophe et homme politique camerounais titulaire d'un doctorat d'État en lettres et sciences humaines de la Sorbonne ainsi que d'une licence en philosophie, un DES, puis son doctorat grâce à une bourse des Nations unies. Enseignant à l'Université de Yaoundé, il a influencé la philosophie africaine contemporaine. &lt;/p&gt; &lt;p&gt; Son premier livre majeur,  &lt;a href="https://www.youtube.com/watch?v=QBTYhXqA14s"  title="De la médiocrité à l’excellence : Le réveil urgent de l’Afrique par Apprnds +"&gt;"De la médiocrité à l’excellence"&lt;/a&gt;  paru en  1970, analyse les obstacles au développement du Cameroun et est étudié au programme de terminale. Parmi ses autres ouvrages figurent "Jalons" paru en 1971," Député de la Nation" en 2002 et des travaux récents sur le transhumanisme comme Elixir ou Lignes rouges "éthiques" de l'intelligence artificielle. &lt;/p&gt; &lt;p&gt; Sa pensée, réflexive et analytique, porte sur le développement humain, la vie quotidienne, l'esprit critique et les défis  &lt;a href="https://www.youtube.com/watch?v=IHwd6B-1RfQ"  title=" Quelle éthique pour le transhumanisme par Ebenezer Njoh Mouelle"&gt;éthiques du transhumanisme&lt;/a&gt;. Il encourage l'effort personnel et une gouvernance globale.  &lt;/p&gt; 
-​</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Eb%C3%A9n%C3%A9zer_Njoh-Mouell%C3%A9"  title=" Wikipedia"&gt;Ebénézer NJOH-MOUELLÉ&lt;/a&gt; (né en 1938) est un philosophe et homme politique camerounais, l’une des figures de la philosophie africaine contemporaine. Formé en France, docteur d’État de la Sorbonne, il enseigne la philosophie à l’université de Yaoundé, où il dirige le département de philosophie et forme plusieurs générations d’étudiants. Il a aussi exercé des responsabilités politiques, notamment comme député à l’Assemblée nationale du Cameroun.&lt;/p&gt; &lt;p&gt;Son livre le plus connu, &lt;a href="https://www.youtube.com/watch?v=QBTYhXqA14s"  title="De la médiocrité à l’excellence : Le réveil urgent de l’Afrique par Apprnds +"&gt;&lt;em&gt;De la médiocrité à l’excellence&lt;/em&gt;&lt;/a&gt; (1970), sous-titré « essai sur la signification humaine du développement », est étudié dans les classes de terminale de plusieurs pays d’Afrique. Njoh-Mouellé y soutient que le développement ne se réduit pas à la croissance économique ou à l’accumulation de biens : il est d’abord l’épanouissement de l’homme tout entier. La médiocrité, c’est se contenter de ce qui est moyen, imiter, se laisser porter ; l’excellence, c’est l’effort pour se dépasser, la liberté créatrice et l’esprit critique. Un peuple ne se développe pas en copiant des modèles venus d’ailleurs, mais en libérant les capacités de création de chacun. Dans &lt;em&gt;Jalons&lt;/em&gt; et ses autres essais, il réfléchit à la place de la philosophie en Afrique, à la tradition, à la modernité et à la responsabilité des intellectuels. Il refuse aussi bien la nostalgie d’un passé idéalisé que l’imitation servile de l’Occident.&lt;/p&gt; &lt;p&gt;Dans ses travaux récents, il s’interroge sur les &lt;a href="https://www.youtube.com/watch?v=IHwd6B-1RfQ"  title=" Quelle éthique pour le transhumanisme par Ebenezer Njoh Mouelle"&gt;enjeux éthiques du transhumanisme&lt;/a&gt; et de l’intelligence artificielle, et sur les limites que l’humanité doit poser aux techniques qui prétendent la transformer.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F14" s="7" t="s">
@@ -4846,8 +4845,11 @@
       <c r="D35" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="E35" s="9" t="s">
-        <v>281</v>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Catherine_Elgin"  title=" Wikipedia"&gt;Catherine ELGIN&lt;/a&gt;   est une philosophe américaine, professeure à Harvard et spécialiste en épistémologie ainsi qu'en esthétique. Elle est  &lt;a href="https://catherineelgin.com/" title=" Catherine Z Elgin"&gt;notamment connue &lt;/a&gt; pour sa longue collaboration avec Nelson Goodman, avec qui elle a exploré les liens entre philosophie, arts et sciences. &lt;/p&gt; &lt;p&gt; Sa philosophie remet en question la quête traditionnelle de la vérité absolue en épistémologie. Pour elle, la compréhension prime sur la connaissance factuelle, car elle permet de saisir des ensembles cohérents et systématiques, même si ceux-ci incluent des modèles idéalisés ou des approximations. &lt;/p&gt; &lt;p&gt; Dans Considered Judgment, elle défend l'équilibre réfléchi comme norme de rationalité : &lt;a href="https://www.youtube.com/watch?v=yqkooYMmVNU" title=" Disagreement between aquals par philosophy Univ Edinburgh"&gt;les croyances &lt;/a&gt;  sont évaluées non par leur correspondance stricte à la réalité, mais par leur cohérence globale et leur capacité à éclairer le monde. &lt;/p&gt; &lt;p&gt; Elle applique cette approche à l'esthétique et aux sciences, où l'art et les fictions servent d'expériences de pensée pour approfondir la compréhension. Sa pensée valorise ainsi une épistémologie flexible, attentive aux valeurs cognitives au-delà des faits bruts. Elle soutient notamment qu’une théorie scientifique peut faire progresser notre compréhension même si elle repose sur des simplifications qui, prises à la lettre, sont fausses : le gaz parfait ou le plan sans frottement sont des « fictions heureuses », qui mettent en évidence ce qui compte. De même, une œuvre d’art nous apprend à voir le monde autrement, en exemplifiant des propriétés que nous n’avions pas remarquées. Avec Goodman, elle a écrit &lt;em&gt;Reconceptions en philosophie&lt;/em&gt; (1988). &lt;/p&gt; 
+</t>
+        </is>
       </c>
       <c r="F35" s="7" t="s">
         <v>282</v>
@@ -5548,8 +5550,10 @@
       <c r="D50" s="8" t="s">
         <v>389</v>
       </c>
-      <c r="E50" s="14" t="s">
-        <v>390</v>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Vandana_Shiva"   title=" Wikipedia"&gt;Vandana SHIVA&lt;/a&gt; est une philosophe indienne, physicienne de formation devenue philosophe des sciences, écoféministe et militante environnementale reconnue mondialement. Elle étudie la physique à l'université du Pendjab, obtient un master puis un doctorat en philosophie des sciences, influencée par sa sœur médecin qui l'alerte sur les risques des radiations. Sa thèse, soutenue au Canada, porte sur les variables cachées en théorie quantique. &lt;/p&gt; &lt;p&gt; En 1982, elle fonde la "Research Foundation for Science, Technology and Natural Resource Policy" pour promouvoir une agriculture durable. En 1991, elle crée &lt;a href="https://www.youtube.com/watch?v=YEqTo8lDivs"  title=" Bande-annonce Les graines de Vandana Shiva  par The Seeds of Vandana Shiva"&gt;Navdanya&lt;/a&gt;, une ONG protégeant la biodiversité agricole indienne contre les OGM et multinationales comme Monsanto. Elle lutte aussi contre les barrages, comme celui de Narmada. &lt;/p&gt; &lt;p&gt; Chef de file de &lt;a href="https://wildproject.org/auteurs/vandana-shiva" title=" Vandana Shiva  par wildproject"&gt;l'écoféminisme&lt;/a&gt;, elle lie oppression des femmes et exploitation de la nature par le néolibéralisme agro-industriel, prônant un retour aux savoirs traditionnels et à la souveraineté alimentaire. Ses ouvrages comme "Staying Alive" paru en 1988 et "Écoféministe" en 1993, repositionnent les femmes comme gardiennes de l'écologie. Elle a été marquée par le mouvement Chipko des années 1970, où des paysannes de l’Himalaya enlaçaient les arbres pour empêcher leur abattage. Elle critique la « révolution verte », qui a imposé en Inde les semences à haut rendement, les engrais chimiques et l’irrigation intensive, et dénonce le brevetage du vivant, qu’elle appelle « biopiraterie ». Elle reçoit en 1993 le prix Nobel alternatif. Ses positions contre les OGM sont toutefois contestées par une partie des scientifiques. &lt;/p&gt; &lt;p&gt; &lt;/p&gt; &lt;p&gt; &lt;p&gt;&lt;/p&gt; &lt;p&gt; &lt;/p&gt; &lt;audio controls title=" Vandana Shiva, les souvenirs d'une femme de combat par France Culture"&gt; &lt;source  src="https://media.radiofrance-podcast.net/podcast09/16410-26.12.2023-ITEMA_23596286-2023C26376E0017-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F50" s="7" t="s">
         <v>391</v>
@@ -6689,8 +6693,7 @@
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Roberto_R._Aramayo" title=" Wikipedia"&gt;Roberto R.ARAMAYO&lt;/a&gt; est un philosophe espagnol, professeur de recherche à l’Institut de Philosophie du CSIC à Madrid. Spécialiste de l’histoire des idées morales et politiques, il dirige le groupe Theoria cum praxi avec Concha Roldán et s’intéresse à l’Illumination européenne. &lt;/p&gt; &lt;p&gt; Sa philosophie cherche à relier théorie et pratique, en étudiant comment les Lumières – chez Rousseau, Kant, Diderot – répondent aux crises et révolutions. Il voit dans ces penseurs une éthique de l’espoir et de l’autonomie qui reste actuelle pour affronter les défis sociaux. &lt;/p&gt; &lt;p&gt; Chez lui, Kant occupe une place centrale : il analyse l’espoir comme une force morale, l’autonomie comme confiance en soi, et le bonheur comme un idéal indépendant de la fortune.   &lt;a href="https://www.youtube.com/watch?v=YkxpcKRgEwg" title="Roberto R Aramayo del intituto Filosofia par CCHSCIC"&gt;Il dialogue aussi &lt;/a&gt; avec Schopenhauer et Cassirer pour penser la justice et la praxis. &lt;/p&gt; &lt;p&gt; On peut donc dire qu’il est un philosophe du pont entre passé et présent. Sa pensée défend la philosophie des Lumières comme un outil vivant pour la démocratie, l’éthique et la transformation sociale. &lt;/p&gt; 
-</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Roberto_R._Aramayo" title=" Wikipedia"&gt;Roberto R. ARAMAYO&lt;/a&gt; (né en 1958) est un philosophe espagnol, professeur de recherche à l’Institut de philosophie du Conseil supérieur de la recherche scientifique (CSIC), à Madrid. Spécialiste de l’histoire des idées morales et politiques, il anime avec Concha Roldán le groupe de recherche &lt;em&gt;Theoria cum praxi&lt;/em&gt;, consacré aux Lumières européennes et à leur actualité.&lt;/p&gt; &lt;p&gt;Il est l’un des grands traducteurs et commentateurs espagnols de Kant, dont il a traduit et présenté de nombreuses œuvres, en particulier ses écrits moraux et politiques, ainsi que de Schopenhauer et de Diderot. Sa philosophie cherche à relier la théorie et la pratique, en étudiant comment les penseurs des Lumières, Rousseau, Diderot ou Kant, ont répondu aux crises et aux révolutions de leur temps. Chez Kant, il s’intéresse surtout à la dimension morale et politique : l’autonomie, la capacité de se donner à soi-même sa propre loi ; l’espérance, qui permet d’agir pour un monde meilleur sans garantie de succès ; et le bonheur, que Kant distingue de la vertu et qui ne doit pas dépendre du hasard ni de la fortune. Il a aussi étudié l’idée du « roi philosophe » et les rapports, souvent difficiles, entre les philosophes et le pouvoir, de Platon aux despotes éclairés. &lt;a href="https://www.youtube.com/watch?v=YkxpcKRgEwg" title="Roberto R Aramayo del intituto Filosofia par CCHSCIC"&gt;Il dialogue aussi&lt;/a&gt; avec Schopenhauer et Cassirer pour penser la justice, l’action politique et le rôle de la philosophie dans la cité.&lt;/p&gt; &lt;p&gt;Pour lui, les Lumières ne sont pas une époque révolue, mais un projet toujours vivant, un outil pour la démocratie, l’éthique et la transformation sociale.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F75" s="7" t="s">
@@ -6917,8 +6920,10 @@
       <c r="D80" s="1" t="s">
         <v>610</v>
       </c>
-      <c r="E80" s="2" t="s">
-        <v>611</v>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Eduardo_Gudynas" title=" Wikipedia (es)"&gt;Eduardo Gudynas&lt;/a&gt; (né en 1960) est un chercheur et essayiste uruguayen, spécialiste de l’écologie politique et l’un des principaux penseurs latino-américains du &lt;em&gt;Buen Vivir&lt;/em&gt;, le « bien-vivre ». Il travaille à Montevideo au Centre latino-américain d’écologie sociale (CLAES), et conseille de nombreux mouvements sociaux.&lt;/p&gt; &lt;p&gt;Le &lt;em&gt;Buen Vivir&lt;/em&gt; s’inspire de notions des peuples andins, le &lt;em&gt;sumak kawsay&lt;/em&gt; des Quechuas et le &lt;em&gt;suma qamaña&lt;/em&gt; des Aymaras, qui désignent une vie pleine, en harmonie avec la communauté et avec la nature. Gudynas en fait une critique de l’idée même de développement : la croissance économique, mesurée par la production de richesses, ne peut être le but d’une société, et le modèle occidental, qui traite la nature comme un réservoir de ressources, mène à l’impasse écologique. Il ne s’agit pas de chercher un « autre développement », mais une alternative au développement. Il est surtout connu pour ses analyses de l’&lt;a href="https://fr.wikipedia.org/wiki/Extractivisme" title=" Wikipedia"&gt;extractivisme&lt;/a&gt; : l’exploitation intensive des mines, du pétrole et des monocultures pour l’exportation. Il montre que les gouvernements de gauche arrivés au pouvoir en Amérique du Sud dans les années 2000 ont prolongé ce modèle, sous une forme qu’il appelle « néo-extractivisme progressiste », en finançant leurs politiques sociales par la destruction de la nature. Il propose des transitions vers un « post-extractivisme ».&lt;/p&gt; &lt;p&gt;Défenseur des droits de la nature, il soutient une éthique biocentrique, qui reconnaît une valeur propre aux êtres vivants. La constitution de l’Équateur (2008), qui reconnaît les droits de la Terre-Mère, et celle de la Bolivie (2009) ont repris ces idées.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F80" s="1" t="s">
         <v>612</v>
@@ -7047,8 +7052,11 @@
       <c r="D83" s="8" t="s">
         <v>633</v>
       </c>
-      <c r="E83" s="11" t="s">
-        <v>634</v>
+      <c r="E83" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://perso.uclouvain.be/marc.maesschalck/index.php" title=" Marc MAESSCHALCK"&gt;Marc MAESSCHALCK&lt;/a&gt;  est un philosophe belge, professeur à l’Université catholique de Louvain. Son travail s’intéresse surtout à la philosophie politique, à l’éthique sociale et à la gouvernance démocratique. &lt;/p&gt; &lt;p&gt; Sa pensée tourne autour d’une idée importante : les normes, la justice et la vie commune ne sont pas fixes, elles se construisent dans des contextes concrets. Il défend une approche contextuelle et pragmatique de l’éthique, où il faut toujours tenir compte des situations réelles, des relations sociales et des formes de coopération. &lt;/p&gt; &lt;p&gt; Il s’intéresse aussi beaucoup à la critique sociale et aux questions décoloniales. Chez lui, penser la société, c’est chercher comment transformer les rapports de pouvoir, ouvrir des espaces de relation plus justes et éviter les formes de domination qui figent les identités ou les légitimités. &lt;/p&gt; &lt;p&gt; On peut donc dire qu’il  est un philosophe de la relation, du collectif et de la transformation. Sa philosophie veut comprendre comment des groupes humains peuvent mieux vivre ensemble, en inventant des normes plus souples, plus démocratiques et plus attentives aux contextes. Spécialiste de Fichte et de la philosophie allemande, auxquels il a consacré ses premiers travaux, il a ensuite développé, au Centre de philosophie du droit de Louvain, une théorie de la gouvernance qui s’interroge sur les conditions dans lesquelles une norme peut réellement transformer les pratiques. Il a aussi travaillé avec des chercheurs d’Amérique latine et d’Afrique sur les mouvements sociaux et les pensées de la libération. &lt;/p&gt; 
+</t>
+        </is>
       </c>
       <c r="F83" s="7" t="s">
         <v>635</v>
@@ -7710,8 +7718,11 @@
       <c r="D98" s="8" t="s">
         <v>748</v>
       </c>
-      <c r="E98" s="9" t="s">
-        <v>749</v>
+      <c r="E98" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Alexander_Schnell" title=" Wikipedia"&gt;Alexander SCHNELL&lt;/a&gt;   est un philosophe  germano-bulgare spécialiste de l'idéalisme allemand (Kant, Fichte, Schelling) et de la phénoménologie (Husserl, Heidegger, Fink, Richir, Lévinas), il publie une trentaine d'ouvrages en français et allemand, comme Husserl et les fondements de la phénoménologie constructive (2007), Was ist Phänomenologie? (2019) ou sa trilogie récente : La déhiscence du sens (2015), Le clignotement de l’être (2021) et Préphénoménalité et générativité (2025). Il traduit aussi des textes philosophiques et édite des volumes collectifs. &lt;/p&gt; &lt;p&gt; Il développe une &lt;a href="https://www.youtube.com/watch?v=PuQPvr3xhEM" title="Prephenomenalité alexxander Schnell et Charles Bobant par Salon Tout Art"&gt;« phénoménologie constructive » &lt;/a&gt; ou « transcendantalisme spéculatif », reprenant le projet husserlien d'une phénoménologie de la connaissance comme idéalisme transcendantal, en intégrant imagination, inconscient phénoménologique, préphénoménalité et générativité. Ses travaux lient philosophie allemande classique, phénoménologie allemande et française, avec des accents sur esthétique et anthropologie, critiquant le primat descriptif au profit de constructions spéculatives. Professeur à l’université de Wuppertal, en Allemagne, après avoir enseigné à Paris-Sorbonne, il veut montrer que la phénoménologie ne se contente pas de décrire ce qui apparaît : elle doit reconstruire les conditions, en deçà de l’apparaître, qui rendent possible le sens. Il prolonge ainsi l’héritage de Fichte et de Marc Richir, dans un dialogue constant entre les traditions française et allemande. &lt;/p&gt; 
+</t>
+        </is>
       </c>
       <c r="F98" s="7" t="s">
         <v>750</v>
@@ -7985,8 +7996,7 @@
       </c>
       <c r="E104" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt; &lt;a href="https://fr.wikipedia.org/wiki/Markus_Gabriel"   title=" Wikipedia"&gt; Markus GABRIEL&lt;/a&gt; est un jeune philosophe Allemand qui est une figure de plus en plus remarquée dans le paysage philosophique mondial. Affirmant une rupture radicale avec la pensée occidentale, il prône un  &lt;a href="https://www.lesinrocks.com/livres/markus-gabriel-existe-excepte-monde-105595-30-09-2014/"   title="Markus Gabriel par les Inrockuptibles"&gt;“nouveau réalisme”&lt;/a&gt;.  &lt;/p&gt; &lt;p&gt; Il s'est fait connaître pour sa théorie de &lt;a href="https://fr.wikipedia.org/wiki/Ontologie_(philosophie)"  title="Ontologie par Wikipédia"&gt;l'ontologie&lt;/a&gt; nouvelle, qui propose une conception nouvelle de la réalité, en opposition à la métaphysique traditionnelle. Selon lui, la réalité n'est pas quelque chose qui existe en soi, indépendamment de notre perception et de notre connaissance, mais plutôt quelque chose qui est créé par notre propre activité cognitive. Autrement dit, la réalité est une construction sociale, qui dépend de notre langage et de notre culture et non de la perception humaine et qui existe indépendamment de notre esprit. &lt;/p&gt; &lt;p&gt; 
-Il a écrit de nombreux livres, dont  « Pourquoi le monde n'existe pas », « Je ne suis pas un cerveau : philosophie de l'esprit pour le 21e siècle » et  &lt;a href="https://www.youtube.com/watch?v=cRxd09vFcxg&amp;ab_channel=FRANCE24"     style="color:#88A1E9"  title="Le pouvoir de l'Art par France 24"&gt;" Le pouvoir de 'Art"&lt;/a&gt;. &lt;/p&gt; &lt;p&gt; Il contribue également régulièrement à divers journaux et magazines et est apparu dans de nombreuses émissions de télévision et de radio pour discuter de ses idées. &lt;/p&gt;   &lt;audio controls title="Si google anticipe pour moi, cela ne veut pas dire qu'il choisit pour moi  par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/16602-10.02.2017-ITEMA_21225836-0.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; &lt;p&gt; &lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Markus_Gabriel"   title=" Wikipedia"&gt;Markus GABRIEL&lt;/a&gt; (né en 1980) est un philosophe allemand, l’un des penseurs les plus en vue de sa génération. Nommé à vingt-neuf ans professeur à l’université de Bonn, ce qui fait de lui le plus jeune titulaire d’une chaire de philosophie en Allemagne, il est spécialiste de l’idéalisme allemand et de la philosophie antique. Il est surtout connu comme l’un des fondateurs, avec l’Italien Maurizio Ferraris, du &lt;a href="https://www.lesinrocks.com/livres/markus-gabriel-existe-excepte-monde-105595-30-09-2014/"   title="Markus Gabriel par les Inrockuptibles"&gt;« nouveau réalisme »&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Contre le constructivisme, pour qui la réalité n’est qu’une construction de notre esprit, de notre langage ou de notre culture, le nouveau réalisme affirme que nous pouvons connaître les choses telles qu’elles sont. Mais Gabriel refuse aussi le naturalisme, qui ne reconnaît comme réel que ce qu’étudient les sciences de la nature. Son &lt;a href="https://fr.wikipedia.org/wiki/Ontologie_(philosophie)"  title="Ontologie par Wikipédia"&gt;ontologie&lt;/a&gt; repose sur la notion de « champ de sens » : exister, c’est apparaître dans un champ de sens. Les montagnes existent dans le champ de la géographie, les nombres dans celui des mathématiques, les licornes dans celui de la fiction. Il existe une infinité de tels champs. En revanche, le monde, compris comme le champ de tous les champs, n’existe pas, car il ne peut apparaître dans aucun champ plus vaste : c’est la thèse provocante de son livre &lt;em&gt;Pourquoi le monde n’existe pas&lt;/em&gt; (2013), devenu un succès international. Dans &lt;em&gt;Je ne suis pas un cerveau&lt;/em&gt; (2015), il critique l’idée que l’esprit se réduirait au cerveau. Il défend aussi un réalisme moral : il existe des faits moraux que nous pouvons connaître.&lt;/p&gt; &lt;p&gt;Il a également écrit sur &lt;a href="https://www.youtube.com/watch?v=cRxd09vFcxg&amp;ab_channel=FRANCE24"     style="color:#88A1E9"  title="Le pouvoir de l'Art par France 24"&gt;le pouvoir de l’art&lt;/a&gt; et intervient souvent dans les médias sur la technique, la démocratie et l’éthique.&lt;/p&gt;  &lt;audio controls title="Si google anticipe pour moi, cela ne veut pas dire qu'il choisit pour moi  par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/16602-10.02.2017-ITEMA_21225836-0.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
       <c r="F104" s="7" t="s">

</xml_diff>